<commit_message>
📊 Horarios actualizados Línea 141 - 1752
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:44:14</t>
+          <t>Última actualización: 02:07:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>00:44:14</t>
+          <t>02:07:51</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:13</t>
+          <t>02:56</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,23 +498,48 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>00:44:14</t>
+          <t>02:07:51</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>01:59</t>
+          <t>03:50</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>83_ESC 6_ALUAR</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>103</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:07:51</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>03:53</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>75</v>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="D8" t="n">
+        <v>106</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -544,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:44:14</t>
+          <t>Última actualización: 02:07:51</t>
         </is>
       </c>
     </row>
@@ -585,12 +610,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>00:44:14</t>
+          <t>02:07:51</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:13</t>
+          <t>02:56</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -599,7 +624,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -631,7 +656,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:44:14</t>
+          <t>Última actualización: 02:07:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1753
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:07:51</t>
+          <t>Última actualización: 03:03:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:07:51</t>
+          <t>03:03:08</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:56</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,12 +498,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:07:51</t>
+          <t>03:03:08</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:50</t>
+          <t>03:51</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>103</v>
+        <v>48</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,12 +523,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:07:51</t>
+          <t>03:03:08</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>03:53</t>
+          <t>04:32</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -537,9 +537,59 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03:03:08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>105</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>03:03:08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>105</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -569,7 +619,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:07:51</t>
+          <t>Última actualización: 03:03:08</t>
         </is>
       </c>
     </row>
@@ -610,21 +660,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:07:51</t>
+          <t>03:03:08</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:56</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>49</v>
+        <v>105</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -656,7 +706,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:07:51</t>
+          <t>Última actualización: 03:03:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1754
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:03:08</t>
+          <t>Última actualización: 04:09:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:03:08</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:32</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:03:08</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:51</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>83_ESC 6_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:03:08</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:32</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>89</v>
+        <v>39</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:03:08</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>05:06</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>105</v>
+        <v>57</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,23 +573,198 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:03:08</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>05:20</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>71</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>04:09:32</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>05:29</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>80</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>04:09:32</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>05:29</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>80</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:09:32</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>81</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:09:32</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>05:32</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>83</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:09:32</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>05:42</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>93</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:09:32</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>05:45</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>96</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:09:32</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>05:48</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>105</v>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="D17" t="n">
+        <v>99</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -606,7 +781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -619,14 +794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:03:08</t>
+          <t>Última actualización: 04:09:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -660,7 +835,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:03:08</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -674,9 +849,59 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>105</v>
+        <v>39</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>04:09:32</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>05:29</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>80</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>04:09:32</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>05:48</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>99</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -693,7 +918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -706,14 +931,91 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:03:08</t>
+          <t>Última actualización: 04:09:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>04:09:32</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>05:29</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>80</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>04:09:32</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06:04</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>115</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1755
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:09:32</t>
+          <t>Última actualización: 04:52:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:06</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:20</t>
+          <t>05:06</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>71</v>
+        <v>14</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:29</t>
+          <t>05:09</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>80</v>
+        <v>17</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05:29</t>
+          <t>05:20</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>80</v>
+        <v>28</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>05:30</t>
+          <t>05:29</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>81</v>
+        <v>37</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>05:32</t>
+          <t>05:29</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>83</v>
+        <v>37</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>05:42</t>
+          <t>05:30</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>93</v>
+        <v>38</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -728,16 +728,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>05:45</t>
+          <t>05:32</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,23 +748,448 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>05:40</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>48</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>05:42</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>50</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>05:45</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>53</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>05:48</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D20" t="n">
+        <v>56</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>68</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>06:14</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>82</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>06:18</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>86</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>06:18</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>86</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>06:21</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>89</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>06:23</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>86XR36_ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>91</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>06:31</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
         <v>99</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>06:34</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>102</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>109</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>109</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>06:44</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>84_ESC AGRARIA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>112</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>06:47</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>11_185Y38_ESC61-ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>115</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>06:50</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>118</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>06:51</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>119</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -781,7 +1206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -794,14 +1219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:09:32</t>
+          <t>Última actualización: 04:52:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -860,7 +1285,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -874,7 +1299,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>80</v>
+        <v>37</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -885,7 +1310,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -899,9 +1324,59 @@
         </is>
       </c>
       <c r="D8" t="n">
+        <v>56</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06:14</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>82</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06:31</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
         <v>99</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -918,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -931,14 +1406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:09:32</t>
+          <t>Última actualización: 04:52:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -972,12 +1447,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:29</t>
+          <t>05:28</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -986,7 +1461,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>80</v>
+        <v>36</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1002,18 +1477,68 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>05:29</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>80</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>06:04</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>115</v>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="D8" t="n">
+        <v>72</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>04:52:36</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06:50</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>118</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1756
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:52:36</t>
+          <t>Última actualización: 05:28:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -683,11 +683,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,7 +698,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>05:40</t>
+          <t>05:32</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>48</v>
+        <v>83</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>05:42</t>
+          <t>05:40</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -803,16 +803,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>05:45</t>
+          <t>05:42</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>05:48</t>
+          <t>05:43</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>56</v>
+        <v>15</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>05:45</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,12 +873,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>06:14</t>
+          <t>05:48</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>82</v>
+        <v>20</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>06:18</t>
+          <t>05:51</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>86</v>
+        <v>23</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,21 +923,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>06:18</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>86</v>
+        <v>32</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,21 +948,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>06:08</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>89</v>
+        <v>40</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,21 +973,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>06:23</t>
+          <t>06:14</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>86XR36_ESC AGRARIA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>91</v>
+        <v>46</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>06:31</t>
+          <t>06:18</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>06:34</t>
+          <t>06:18</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>102</v>
+        <v>50</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>06:21</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>109</v>
+        <v>53</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1078,16 +1078,16 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>06:23</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>06:44</t>
+          <t>06:24</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>84_ESC AGRARIA-ESC 49</t>
+          <t>86XR36_ESC AGRARIA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>112</v>
+        <v>56</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>06:47</t>
+          <t>06:31</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>11_185Y38_ESC61-ETCHEVERRY</t>
+          <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>115</v>
+        <v>63</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>06:50</t>
+          <t>06:34</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>118</v>
+        <v>66</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,23 +1173,348 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>73</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>73</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>06:44</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>84_ESC AGRARIA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>76</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>06:47</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>11_185Y38_ESC61-ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>79</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>06:50</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>82</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
           <t>06:51</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>119</v>
-      </c>
-      <c r="E34" t="inlineStr">
+      <c r="D39" t="n">
+        <v>83</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>06:58</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>10_ESC70-OLMOS</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>90</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>07:03</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>17/64_OLMOS POR 520</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>95</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>07:07</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>99</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>07:13</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>105</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>107</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>112</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>113</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>07:26</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>118</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1206,7 +1531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1219,14 +1544,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:52:36</t>
+          <t>Última actualización: 05:28:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1310,21 +1635,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:48</t>
+          <t>05:32</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>56</v>
+        <v>4</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1335,12 +1660,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06:14</t>
+          <t>05:48</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1349,7 +1674,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>82</v>
+        <v>20</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1360,23 +1685,73 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>06:14</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>46</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>06:31</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>99</v>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="D11" t="n">
+        <v>63</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>107</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1393,7 +1768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1406,14 +1781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:52:36</t>
+          <t>Última actualización: 05:28:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1847,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1486,7 +1861,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1497,7 +1872,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1511,7 +1886,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1539,6 +1914,81 @@
         <v>118</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06:51</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>83</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06:53</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>85</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>05:28:28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>114</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1757
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:28:28</t>
+          <t>Última actualización: 06:05:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 42</t>
+          <t>Total filas: 54</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -948,7 +948,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>46</v>
+        <v>9</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1008,11 +1008,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>53</v>
+        <v>16</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>63</v>
+        <v>26</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>66</v>
+        <v>29</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>73</v>
+        <v>36</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>73</v>
+        <v>36</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,7 +1223,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>79</v>
+        <v>42</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>83</v>
+        <v>46</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>90</v>
+        <v>53</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1362,7 +1362,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>95</v>
+        <v>58</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>99</v>
+        <v>62</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07:13</t>
+          <t>07:08</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>105</v>
+        <v>63</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>07:13</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>107</v>
+        <v>68</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>112</v>
+        <v>70</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>113</v>
+        <v>75</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,23 +1498,323 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>76</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>76</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>07:26</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D47" t="n">
-        <v>118</v>
-      </c>
-      <c r="E47" t="inlineStr">
+      <c r="D49" t="n">
+        <v>81</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>07:29</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>84</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>87</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>07:32</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>87</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>91</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>07:38</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>93</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>105</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>106</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>07:56</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>111</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>115</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>08:02</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>117</v>
+      </c>
+      <c r="E59" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1531,7 +1831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1544,14 +1844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:28:28</t>
+          <t>Última actualización: 06:05:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1985,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1699,7 +1999,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>46</v>
+        <v>9</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1710,7 +2010,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1724,7 +2024,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>63</v>
+        <v>26</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1735,7 +2035,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1749,9 +2049,34 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>107</v>
+        <v>70</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>07:29</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>84</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1768,7 +2093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1781,14 +2106,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:28:28</t>
+          <t>Última actualización: 06:05:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1897,21 +2222,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06:50</t>
+          <t>06:06</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>118</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1922,12 +2247,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:51</t>
+          <t>06:50</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1936,7 +2261,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>83</v>
+        <v>45</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1952,43 +2277,68 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:53</t>
+          <t>06:51</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215D_LA PLATA</t>
+          <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>06:53</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>48</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>07:22</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>114</v>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="D13" t="n">
+        <v>77</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1758
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:05:16</t>
+          <t>Última actualización: 06:55:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 54</t>
+          <t>Total filas: 73</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1323,12 +1323,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>06:58</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1353,16 +1353,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>07:03</t>
+          <t>06:58</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>10_ESC70-OLMOS</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>07:07</t>
+          <t>07:03</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>62</v>
+        <v>8</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07:08</t>
+          <t>07:07</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>63</v>
+        <v>12</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>07:13</t>
+          <t>07:08</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>68</v>
+        <v>13</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1453,16 +1453,16 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>07:08</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:13</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:14</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>76</v>
+        <v>19</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,21 +1523,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:15</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>81</v>
+        <v>25</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1578,16 +1578,16 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>87</v>
+        <v>26</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:24</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>87</v>
+        <v>29</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>91</v>
+        <v>31</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>07:38</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>93</v>
+        <v>34</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,21 +1698,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>07:50</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>105</v>
+        <v>36</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>07:51</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>106</v>
+        <v>37</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>07:56</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>111</v>
+        <v>37</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1778,16 +1778,16 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>115</v>
+        <v>91</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,23 +1798,498 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>07:38</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>43</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>07:42</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>47</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>55</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>56</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>60</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>06:05:16</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>07:56</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>111</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>07:59</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>64</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>06:05:16</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>115</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
         <is>
           <t>08:02</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D59" t="n">
+      <c r="D67" t="n">
+        <v>67</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>08:08</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>73</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>80</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>86</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>86</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>08:24</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>89</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>08:31</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>96</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>98</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>08:36</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>101</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>106</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>08:50</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>115</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>08:52</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
         <v>117</v>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E78" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1831,7 +2306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1844,14 +2319,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:05:16</t>
+          <t>Última actualización: 06:55:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2510,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2049,7 +2524,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2060,7 +2535,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2074,9 +2549,109 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>84</v>
+        <v>34</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>86</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>08:31</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>96</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>98</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>106</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2093,7 +2668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2106,14 +2681,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:05:16</t>
+          <t>Última actualización: 06:55:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2897,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2336,9 +2911,84 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>07:54</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>59</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>08:17</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>82</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>08:52</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>117</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1759
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:55:38</t>
+          <t>Última actualización: 07:27:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 73</t>
+          <t>Total filas: 94</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,12 +1698,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,12 +1723,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>07:32</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>91</v>
+        <v>34</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>07:38</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>43</v>
+        <v>2</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1828,16 +1828,16 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>07:42</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>07:50</t>
+          <t>07:31</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>55</v>
+        <v>4</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>07:51</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>56</v>
+        <v>5</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1903,16 +1903,16 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,12 +1923,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>07:56</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>111</v>
+        <v>37</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>64</v>
+        <v>91</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>115</v>
+        <v>10</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2003,16 +2003,16 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>08:02</t>
+          <t>07:38</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>67</v>
+        <v>43</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,12 +2023,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>08:08</t>
+          <t>07:38</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>73</v>
+        <v>11</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>07:42</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>80</v>
+        <v>15</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>07:50</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>86</v>
+        <v>23</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>07:51</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>86</v>
+        <v>24</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>08:24</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>08:31</t>
+          <t>07:56</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>08:33</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>98</v>
+        <v>32</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>08:36</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:02</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>106</v>
+        <v>35</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>08:50</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>115</v>
+        <v>36</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2278,18 +2278,543 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
+          <t>08:08</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>73</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>48</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>08:20</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>53</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>08:20</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>53</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>86</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>86</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>54</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>08:23</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>56</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>08:24</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>89</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>08:31</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>64</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>08:32</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>65</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>98</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>08:36</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>101</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>08:40</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>73</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>106</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>08:50</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>83</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>08:51</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>84</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
           <t>08:52</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D78" t="n">
+      <c r="D95" t="n">
         <v>117</v>
       </c>
-      <c r="E78" t="inlineStr">
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>09:13</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>106</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>112</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>113</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>113</v>
+      </c>
+      <c r="E99" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2306,7 +2831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2319,14 +2844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:55:38</t>
+          <t>Última actualización: 07:27:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -2535,12 +3060,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2549,7 +3074,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2565,16 +3090,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>86</v>
+        <v>34</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2585,21 +3110,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>08:31</t>
+          <t>08:20</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>96</v>
+        <v>53</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2615,16 +3140,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>08:33</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2635,23 +3160,148 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>08:31</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>64</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>08:32</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>65</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>06:55:38</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>98</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08:40</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>73</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>06:55:38</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>08:41</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D21" t="n">
         <v>106</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>113</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2668,7 +3318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2681,14 +3331,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:55:38</t>
+          <t>Última actualización: 07:27:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2922,7 +3572,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2936,7 +3586,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2947,48 +3597,73 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>08:17</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>50</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>08:52</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>117</v>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="D17" t="n">
+        <v>85</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1760
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:E120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:27:56</t>
+          <t>Última actualización: 08:03:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 94</t>
+          <t>Total filas: 115</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2273,21 +2273,21 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>08:08</t>
+          <t>08:05</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>73</v>
+        <v>2</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>08:08</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>48</v>
+        <v>5</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>08:20</t>
+          <t>08:09</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>53</v>
+        <v>6</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>08:20</t>
+          <t>08:12</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>53</v>
+        <v>9</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:15</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>86</v>
+        <v>12</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>86</v>
+        <v>16</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2428,16 +2428,16 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:20</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2453,16 +2453,16 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>08:23</t>
+          <t>08:20</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>08:24</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>89</v>
+        <v>18</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2503,16 +2503,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>08:31</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>08:32</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>08:33</t>
+          <t>08:22</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>98</v>
+        <v>19</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,12 +2573,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>08:36</t>
+          <t>08:22</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>101</v>
+        <v>19</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2603,16 +2603,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>08:40</t>
+          <t>08:23</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:24</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>106</v>
+        <v>21</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,21 +2648,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>08:50</t>
+          <t>08:29</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>83</v>
+        <v>26</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>08:51</t>
+          <t>08:31</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>08:52</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>117</v>
+        <v>65</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>09:13</t>
+          <t>08:33</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>106</v>
+        <v>30</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,21 +2748,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>08:36</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>09:20</t>
+          <t>08:37</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>113</v>
+        <v>34</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2803,18 +2803,543 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
+          <t>08:40</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>73</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>38</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>08:43</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>40</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>08:50</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>47</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>08:51</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>84</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>08:52</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>49</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>09:13</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>106</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>71</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>71</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>71</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>76</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
           <t>09:20</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C110" t="inlineStr">
         <is>
           <t>215D_EL PATO</t>
         </is>
       </c>
-      <c r="D99" t="n">
+      <c r="D110" t="n">
         <v>113</v>
       </c>
-      <c r="E99" t="inlineStr">
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>113</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>78</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>78</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>09:22</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>79</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>84</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>85</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>09:33</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>90</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>09:41</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>98</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>114</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>118</v>
+      </c>
+      <c r="E120" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2831,7 +3356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2844,14 +3369,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:27:56</t>
+          <t>Última actualización: 08:03:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -3135,7 +3660,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3149,7 +3674,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3160,7 +3685,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3174,7 +3699,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3210,7 +3735,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3224,7 +3749,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3260,7 +3785,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3274,7 +3799,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>106</v>
+        <v>38</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3302,6 +3827,81 @@
         <v>113</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>78</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>09:41</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>98</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>114</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3318,7 +3918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3331,14 +3931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:27:56</t>
+          <t>Última actualización: 08:03:22</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -3597,7 +4197,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3611,7 +4211,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>45</v>
+        <v>9</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -3647,23 +4247,73 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>08:18</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>15</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>08:52</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>85</v>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="D18" t="n">
+        <v>49</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>09:23</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>80</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1761
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E120"/>
+  <dimension ref="A1:E141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:03:22</t>
+          <t>Última actualización: 08:40:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 115</t>
+          <t>Total filas: 136</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -658,11 +658,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -683,11 +683,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:40</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>08:43</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>08:50</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>08:51</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>08:52</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>09:13</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>106</v>
+        <v>3</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2978,16 +2978,16 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>08:50</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>71</v>
+        <v>11</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,21 +3048,21 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>08:52</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>76</v>
+        <v>12</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>09:20</t>
+          <t>08:54</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>113</v>
+        <v>14</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>09:20</t>
+          <t>08:58</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>113</v>
+        <v>18</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:01</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>78</v>
+        <v>21</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>78</v>
+        <v>27</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>09:22</t>
+          <t>09:13</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>79</v>
+        <v>106</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>09:27</t>
+          <t>09:14</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>09:28</t>
+          <t>09:14</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>85</v>
+        <v>34</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>09:33</t>
+          <t>09:14</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>90</v>
+        <v>34</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>98</v>
+        <v>39</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3303,16 +3303,16 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>114</v>
+        <v>76</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,23 +3323,548 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>39</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>113</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>40</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>07:27:56</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>113</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>41</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>09:21</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>41</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
           <t>08:03:22</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr">
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>09:22</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>79</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>09:23</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>43</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>84</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>48</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>09:33</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>90</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>54</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>08:03:22</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>09:41</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>98</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>77</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
         <is>
           <t>10:01</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr">
+      <c r="C134" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D120" t="n">
-        <v>118</v>
-      </c>
-      <c r="E120" t="inlineStr">
+      <c r="D134" t="n">
+        <v>81</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>87</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>87</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>91</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>101</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>101</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>107</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>113</v>
+      </c>
+      <c r="E141" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3356,7 +3881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3369,14 +3894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:03:22</t>
+          <t>Última actualización: 08:40:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -3785,7 +4310,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3799,7 +4324,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3835,7 +4360,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3849,7 +4374,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3885,7 +4410,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3899,9 +4424,59 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>114</v>
+        <v>77</v>
       </c>
       <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>91</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>113</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3918,7 +4493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3931,14 +4506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:03:22</t>
+          <t>Última actualización: 08:40:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -4297,23 +4872,148 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>08:53</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>13</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>08:03:22</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>09:23</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D20" t="n">
         <v>80</v>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>44</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>10:05</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>85</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>93</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>10:39</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>119</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1762
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E141"/>
+  <dimension ref="A1:E154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:40:05</t>
+          <t>Última actualización: 08:58:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 136</t>
+          <t>Total filas: 149</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -658,11 +658,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -683,11 +683,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>18</v>
+        <v>86</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>09:01</t>
+          <t>08:59</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>08:59</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>09:13</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>106</v>
+        <v>2</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>71</v>
+        <v>2</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>09:01</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,12 +3273,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:13</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>76</v>
+        <v>106</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:14</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>09:20</t>
+          <t>09:14</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>113</v>
+        <v>16</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>09:20</t>
+          <t>09:14</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>09:20</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>113</v>
+        <v>20</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3428,16 +3428,16 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>09:21</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>09:22</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>79</v>
+        <v>39</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>09:23</t>
+          <t>09:20</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>09:27</t>
+          <t>09:20</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>84</v>
+        <v>113</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3553,16 +3553,16 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>09:28</t>
+          <t>09:20</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>09:33</t>
+          <t>09:20</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:21</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:21</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>98</v>
+        <v>23</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:22</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>77</v>
+        <v>24</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3678,16 +3678,16 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>09:23</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>81</v>
+        <v>43</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>10:07</t>
+          <t>09:27</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>10:07</t>
+          <t>09:28</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>87</v>
+        <v>30</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>09:33</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>91</v>
+        <v>35</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3778,16 +3778,16 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>10:21</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>101</v>
+        <v>54</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>10:21</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>101</v>
+        <v>43</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>107</v>
+        <v>45</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,23 +3848,348 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>09:43</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>45</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>59</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>63</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>69</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>69</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>73</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>83</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>83</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>88</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
           <t>08:40:05</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr">
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>107</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
         <is>
           <t>10:33</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr">
+      <c r="C151" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D141" t="n">
-        <v>113</v>
-      </c>
-      <c r="E141" t="inlineStr">
+      <c r="D151" t="n">
+        <v>95</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>102</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>10:54</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>17/64_OLMOS POR 520</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>116</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>117</v>
+      </c>
+      <c r="E154" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3894,7 +4219,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:40:05</t>
+          <t>Última actualización: 08:58:21</t>
         </is>
       </c>
     </row>
@@ -4360,7 +4685,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4374,7 +4699,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4385,7 +4710,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4399,7 +4724,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>98</v>
+        <v>43</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4410,7 +4735,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4424,7 +4749,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4435,7 +4760,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4449,7 +4774,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4460,7 +4785,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4474,7 +4799,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4493,7 +4818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4506,14 +4831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:40:05</t>
+          <t>Última actualización: 08:58:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -4897,7 +5222,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4911,7 +5236,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -4947,12 +5272,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>10:05</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -4961,7 +5286,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4977,43 +5302,93 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10:13</t>
+          <t>10:05</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-LA PLATA</t>
+          <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>75</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>10:38</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>100</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>08:40:05</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>10:39</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D26" t="n">
         <v>119</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1763
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E154"/>
+  <dimension ref="A1:E194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:58:21</t>
+          <t>Última actualización: 09:53:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 149</t>
+          <t>Total filas: 189</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1608,11 +1608,11 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>26</v>
+        <v>76</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>18</v>
+        <v>86</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>113</v>
+        <v>40</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:53</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,12 +3898,12 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>10:07</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>10:07</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>73</v>
+        <v>2</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>10:21</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>83</v>
+        <v>3</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4028,16 +4028,16 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>10:21</t>
+          <t>09:57</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>83</v>
+        <v>59</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4053,16 +4053,16 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>10:02</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>107</v>
+        <v>9</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>10:33</t>
+          <t>10:06</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>95</v>
+        <v>13</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>10:06</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>102</v>
+        <v>13</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4153,16 +4153,16 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>10:54</t>
+          <t>10:07</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>116</v>
+        <v>69</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4178,18 +4178,1018 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>69</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>17</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>17</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>18</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>73</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>27</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>27</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>83</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>83</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>33</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>08:40:05</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>107</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>10:31</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>38</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>39</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>40</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>95</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>102</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>50</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>10:54</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>17/64_OLMOS POR 520</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>61</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
           <t>10:55</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
+      <c r="C172" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D154" t="n">
-        <v>117</v>
-      </c>
-      <c r="E154" t="inlineStr">
+      <c r="D172" t="n">
+        <v>62</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>65</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>67</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>11:01</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>68</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>69</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>73</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>73</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>75</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>11:11</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>78</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>10_ESC70-OLMOS</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>82</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>11:17</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>84</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>11:18</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>85</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>87</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>11:22</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>89</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>90</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>11:29</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>96</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>11:31</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>98</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>105</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>108</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>109</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>11:48</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>115</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>11:49</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>10_RUTA 36_ESC 70</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>116</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>11:52</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>119</v>
+      </c>
+      <c r="E194" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4206,7 +5206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4219,14 +5219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:58:21</t>
+          <t>Última actualización: 09:53:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -4735,12 +5735,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -4749,7 +5749,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>59</v>
+        <v>3</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4765,16 +5765,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>09:57</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4785,23 +5785,198 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>17</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>08:58:21</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>73</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>39</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>08:58:21</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>10:33</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D30" t="n">
         <v>95</v>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>11:17</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>84</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>11:29</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>96</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>11:31</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>98</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>109</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4818,7 +5993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4831,14 +6006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:58:21</t>
+          <t>Última actualización: 09:53:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -5272,7 +6447,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -5286,7 +6461,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>66</v>
+        <v>11</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -5322,12 +6497,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10:13</t>
+          <t>10:12</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -5336,7 +6511,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>75</v>
+        <v>19</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -5352,43 +6527,118 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10:38</t>
+          <t>10:13</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>10:38</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>45</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>08:40:05</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>10:39</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D27" t="n">
         <v>119</v>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>67</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>99</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1764
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E194"/>
+  <dimension ref="A1:E228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:53:56</t>
+          <t>Última actualización: 10:53:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 189</t>
+          <t>Total filas: 223</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>26</v>
+        <v>76</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1608,11 +1608,11 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>22</v>
+        <v>113</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>113</v>
+        <v>40</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4248,7 +4248,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4258,11 +4258,11 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>95</v>
+        <v>40</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>10:54</t>
+          <t>10:53</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:54</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>62</v>
+        <v>1</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>10:58</t>
+          <t>10:54</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>65</v>
+        <v>1</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:54</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>67</v>
+        <v>1</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>11:01</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4728,16 +4728,16 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>11:02</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>11:06</t>
+          <t>10:58</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>73</v>
+        <v>5</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4778,16 +4778,16 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>11:06</t>
+          <t>10:58</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>10:59</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>75</v>
+        <v>6</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4828,16 +4828,16 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>11:11</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>11:01</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>10_ESC70-OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>82</v>
+        <v>8</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>11:17</t>
+          <t>11:01</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>84</v>
+        <v>8</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4903,16 +4903,16 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>11:18</t>
+          <t>11:02</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>11:03</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>87</v>
+        <v>10</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>11:22</t>
+          <t>11:06</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4978,16 +4978,16 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>11:23</t>
+          <t>11:06</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>11:29</t>
+          <t>11:07</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>96</v>
+        <v>14</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5028,16 +5028,16 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>11:31</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>98</v>
+        <v>75</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:09</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>105</v>
+        <v>16</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5078,16 +5078,16 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>11:41</t>
+          <t>11:11</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>108</v>
+        <v>78</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>11:42</t>
+          <t>11:12</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>109</v>
+        <v>19</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5128,16 +5128,16 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>11:48</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_ESC70-OLMOS</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>115</v>
+        <v>82</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>11:49</t>
+          <t>11:16</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>10_ESC70-OLMOS</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>116</v>
+        <v>23</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5178,18 +5178,868 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
+          <t>11:17</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>84</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>11:18</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>85</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>11:18</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>25</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>26</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>87</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>28</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>11:22</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>89</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>90</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>11:23</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>30</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>11:26</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>33</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>11:29</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>36</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>11:31</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>98</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>11:31</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>38</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>39</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>41</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>45</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>108</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>109</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>11:43</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>50</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>53</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>11:48</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>55</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>11:49</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>10_RUTA 36_ESC 70</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>116</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
           <t>11:52</t>
         </is>
       </c>
-      <c r="C194" t="inlineStr">
+      <c r="C216" t="inlineStr">
         <is>
           <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
-      <c r="D194" t="n">
-        <v>119</v>
-      </c>
-      <c r="E194" t="inlineStr">
+      <c r="D216" t="n">
+        <v>59</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>62</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>65</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>12:02</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>69</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>72</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>77</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>12:21</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>88</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>12:23</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>10_RUTA 36_ESC 70</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>90</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>92</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>99</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>100</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>105</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>12:49</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>116</v>
+      </c>
+      <c r="E228" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5206,7 +6056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5219,14 +6069,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:53:56</t>
+          <t>Última actualización: 10:53:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -5910,21 +6760,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>11:29</t>
+          <t>11:18</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>96</v>
+        <v>25</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5935,21 +6785,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>11:31</t>
+          <t>11:29</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>98</v>
+        <v>36</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5965,18 +6815,118 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>11:31</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>98</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>39</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>09:53:56</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>11:42</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="D36" t="n">
         <v>109</v>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>11:43</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>50</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>72</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5993,7 +6943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6006,14 +6956,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:53:56</t>
+          <t>Última actualización: 10:53:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -6597,12 +7547,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -6611,7 +7561,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>67</v>
+        <v>2</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -6627,18 +7577,93 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>67</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>11:32</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>99</v>
-      </c>
-      <c r="E29" t="inlineStr">
+      <c r="D30" t="n">
+        <v>39</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>72</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>12:18</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>85</v>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1765
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E228"/>
+  <dimension ref="A1:E250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:53:21</t>
+          <t>Última actualización: 11:35:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 223</t>
+          <t>Total filas: 245</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3358,7 +3358,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>113</v>
+        <v>40</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>22</v>
+        <v>113</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>95</v>
+        <v>40</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5208,11 +5208,11 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>11:41</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>11:42</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>109</v>
+        <v>0</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>11:43</t>
+          <t>11:36</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>11:46</t>
+          <t>11:36</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>11:48</t>
+          <t>11:36</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>11:49</t>
+          <t>11:36</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>116</v>
+        <v>1</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>11:37</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>59</v>
+        <v>2</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5753,16 +5753,16 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:38</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,12 +5773,12 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:40</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -5787,7 +5787,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>12:02</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>69</v>
+        <v>108</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>11:42</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>72</v>
+        <v>109</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>12:10</t>
+          <t>11:43</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>77</v>
+        <v>8</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>11:46</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>11:48</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>90</v>
+        <v>13</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>11:48</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>92</v>
+        <v>13</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>11:49</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_RUTA 36_ESC 70</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>99</v>
+        <v>116</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>105</v>
+        <v>20</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,23 +6023,573 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>11:57</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>22</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
           <t>10:53:20</t>
         </is>
       </c>
-      <c r="B228" t="inlineStr">
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>65</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>12:02</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>27</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>29</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>72</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>33</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>35</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>38</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>12:18</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>43</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>12:21</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>46</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>12:23</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>10_RUTA 36_ESC 70</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>90</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>50</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>99</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>100</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>61</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>105</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
         <is>
           <t>12:49</t>
         </is>
       </c>
-      <c r="C228" t="inlineStr">
+      <c r="C244" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D228" t="n">
-        <v>116</v>
-      </c>
-      <c r="E228" t="inlineStr">
+      <c r="D244" t="n">
+        <v>74</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>82</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>10_RUTA 36_ESC 70</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>90</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>13:07</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>92</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>13:07</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>92</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>106</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>110</v>
+      </c>
+      <c r="E250" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6056,7 +6606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6069,14 +6619,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:53:21</t>
+          <t>Última actualización: 11:35:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -6885,7 +7435,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6899,7 +7449,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6910,23 +7460,73 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>29</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>10:53:20</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>12:05</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D39" t="n">
         <v>72</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>61</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6943,7 +7543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6956,14 +7556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:53:21</t>
+          <t>Última actualización: 11:35:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -7622,12 +8222,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -7636,7 +8236,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -7652,20 +8252,170 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>72</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12:17</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>42</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>12:18</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D32" t="n">
+      <c r="D34" t="n">
         <v>85</v>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>87</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>13:10</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>95</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>99</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>13:26</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>111</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1766
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E250"/>
+  <dimension ref="A1:E279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:35:43</t>
+          <t>Última actualización: 12:24:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 245</t>
+          <t>Total filas: 274</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,7 +4748,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -4758,11 +4758,11 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>5</v>
+        <v>65</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4858,7 +4858,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5458,11 +5458,11 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5483,11 +5483,11 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>105</v>
+        <v>1</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,21 +6423,21 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>12:49</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>82</v>
+        <v>1</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>90</v>
+        <v>1</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,21 +6498,21 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>13:07</t>
+          <t>12:26</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,21 +6523,21 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>13:07</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>92</v>
+        <v>5</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,21 +6548,21 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>106</v>
+        <v>6</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,23 +6573,748 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>99</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>100</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>12</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
           <t>11:35:43</t>
         </is>
       </c>
-      <c r="B250" t="inlineStr">
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>61</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>12:37</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>13</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>10:53:20</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>105</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>16</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>12:49</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>25</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>33</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>39</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>41</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>10_RUTA 36_ESC 70</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>90</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>13:07</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>43</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>13:07</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>92</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>11:35:43</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>13:07</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>92</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>49</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>57</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
         <is>
           <t>13:25</t>
         </is>
       </c>
-      <c r="C250" t="inlineStr">
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>61</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D250" t="n">
-        <v>110</v>
-      </c>
-      <c r="E250" t="inlineStr">
+      <c r="D268" t="n">
+        <v>61</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>13:29</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>65</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>13:36</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>72</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>73</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>13:42</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>78</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>92</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>92</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>94</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>14:01</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>97</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>14:02</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>98</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>99</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>14:22</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>118</v>
+      </c>
+      <c r="E279" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6606,7 +7331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6619,14 +7344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:35:43</t>
+          <t>Última actualización: 12:24:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -7527,6 +8252,81 @@
         <v>61</v>
       </c>
       <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>12:37</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>13</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>61</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>99</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7543,7 +8343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7556,14 +8356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:35:43</t>
+          <t>Última actualización: 12:24:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -8347,25 +9147,25 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>13:10</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
@@ -8377,16 +9177,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>13:10</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -8397,25 +9197,125 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>13:14</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>50</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>51</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>11:35:43</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>13:26</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>215C_ESC AGRARIA-LA PLATA</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D40" t="n">
         <v>111</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>13:27</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>63</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>13:42</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>78</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1767
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E279"/>
+  <dimension ref="A1:E301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:24:25</t>
+          <t>Última actualización: 13:01:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 274</t>
+          <t>Total filas: 296</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -658,11 +658,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -683,11 +683,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>18</v>
+        <v>86</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>22</v>
+        <v>113</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4248,7 +4248,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4258,11 +4258,11 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5208,11 +5208,11 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6798,21 +6798,21 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>13:03</t>
+          <t>13:02</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,12 +6823,12 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>13:02</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -6837,7 +6837,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,21 +6848,21 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,21 +6873,21 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>13:07</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6903,16 +6903,16 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>13:07</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>10_RUTA 36_ESC 70</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,21 +6923,21 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>13:07</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>92</v>
+        <v>4</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,21 +6948,21 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>13:07</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>49</v>
+        <v>92</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:07</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>57</v>
+        <v>6</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,21 +6998,21 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:07</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>61</v>
+        <v>92</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,21 +7023,21 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7053,16 +7053,16 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>13:29</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,21 +7073,21 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>13:36</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,21 +7098,21 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>13:37</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,21 +7123,21 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>13:42</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>78</v>
+        <v>23</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7153,16 +7153,16 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>92</v>
+        <v>61</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,21 +7173,21 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,21 +7198,21 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>13:58</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>94</v>
+        <v>24</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,21 +7223,21 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>14:01</t>
+          <t>13:26</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>97</v>
+        <v>25</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>14:02</t>
+          <t>13:28</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>98</v>
+        <v>27</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>13:29</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>99</v>
+        <v>28</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,23 +7298,573 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>13:29</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>28</v>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>34</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
           <t>12:24:25</t>
         </is>
       </c>
-      <c r="B279" t="inlineStr">
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>13:36</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>72</v>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>36</v>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>13:42</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>41</v>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>13:46</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>45</v>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>52</v>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>92</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>92</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>57</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>14:01</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>60</v>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>14:02</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>98</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>62</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>62</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>72</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>80</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
         <is>
           <t>14:22</t>
         </is>
       </c>
-      <c r="C279" t="inlineStr">
+      <c r="C295" t="inlineStr">
         <is>
           <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
-      <c r="D279" t="n">
-        <v>118</v>
-      </c>
-      <c r="E279" t="inlineStr">
+      <c r="D295" t="n">
+        <v>81</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>14:23</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>82</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>92</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>101</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>102</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>109</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>14:51</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>110</v>
+      </c>
+      <c r="E301" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7331,7 +7881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7344,14 +7894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:24:25</t>
+          <t>Última actualización: 13:01:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -8285,12 +8835,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -8299,7 +8849,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>61</v>
+        <v>23</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8315,18 +8865,68 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>61</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>14:03</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>99</v>
-      </c>
-      <c r="E43" t="inlineStr">
+      <c r="D44" t="n">
+        <v>62</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>102</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8343,7 +8943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8356,14 +8956,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:24:25</t>
+          <t>Última actualización: 13:01:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -9122,7 +9722,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -9136,7 +9736,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>87</v>
+        <v>1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -9197,7 +9797,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -9211,7 +9811,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -9247,37 +9847,37 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>13:26</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>111</v>
+        <v>23</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>13:27</t>
+          <t>13:26</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -9286,7 +9886,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -9302,18 +9902,68 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>13:27</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>63</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>12:24:25</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>13:42</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D43" t="n">
         <v>78</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>13:46</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>45</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1768
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E301"/>
+  <dimension ref="A1:E327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:01:41</t>
+          <t>Última actualización: 13:58:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 296</t>
+          <t>Total filas: 322</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -658,11 +658,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -683,11 +683,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1608,11 +1608,11 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>26</v>
+        <v>76</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>18</v>
+        <v>86</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,7 +4748,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -4758,11 +4758,11 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>5</v>
+        <v>65</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5208,11 +5208,11 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5458,11 +5458,11 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5483,11 +5483,11 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D223" t="n">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6898,7 +6898,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -6908,11 +6908,11 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6933,11 +6933,11 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_RUTA 36_ESC 70</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,7 +6948,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -6958,11 +6958,11 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>92</v>
+        <v>6</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,7 +6973,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -6983,11 +6983,11 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>6</v>
+        <v>92</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -7023,7 +7023,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -7033,11 +7033,11 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,7 +7048,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -7058,11 +7058,11 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7158,11 +7158,11 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,7 +7173,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -7183,11 +7183,11 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7283,7 +7283,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D278" t="n">
@@ -7308,7 +7308,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D279" t="n">
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7537,7 +7537,7 @@
         </is>
       </c>
       <c r="D288" t="n">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,21 +7548,21 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>14:01</t>
+          <t>13:59</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>14:02</t>
+          <t>13:59</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>98</v>
+        <v>1</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,21 +7598,21 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>13:59</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>62</v>
+        <v>1</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,21 +7623,21 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,21 +7648,21 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>14:13</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>72</v>
+        <v>3</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,21 +7673,21 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>14:21</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7703,16 +7703,16 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>14:22</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,21 +7723,21 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>14:23</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>82</v>
+        <v>5</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:09</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>92</v>
+        <v>11</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,21 +7773,21 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>14:42</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>101</v>
+        <v>14</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:13</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>102</v>
+        <v>15</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,21 +7823,21 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>109</v>
+        <v>19</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,23 +7848,673 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>20</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>23</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>14:22</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>24</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>14:23</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>25</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>35</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>43</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
           <t>13:01:41</t>
         </is>
       </c>
-      <c r="B301" t="inlineStr">
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>101</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>45</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>13:01:41</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>109</v>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
         <is>
           <t>14:51</t>
         </is>
       </c>
-      <c r="C301" t="inlineStr">
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>53</v>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>14:51</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
         <is>
           <t>83_ALUAR</t>
         </is>
       </c>
-      <c r="D301" t="n">
-        <v>110</v>
-      </c>
-      <c r="E301" t="inlineStr">
+      <c r="D311" t="n">
+        <v>53</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>61</v>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
+        <v>61</v>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>63</v>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>15:03</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D315" t="n">
+        <v>65</v>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>15:08</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D316" t="n">
+        <v>70</v>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>15:12</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>74</v>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>80</v>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>80</v>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>15:21</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D320" t="n">
+        <v>83</v>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>92</v>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>15:33</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D322" t="n">
+        <v>95</v>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>15:37</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>99</v>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>15:43</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D324" t="n">
+        <v>105</v>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D325" t="n">
+        <v>106</v>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>15:49</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D326" t="n">
+        <v>111</v>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>15:49</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D327" t="n">
+        <v>111</v>
+      </c>
+      <c r="E327" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7881,7 +8531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7894,14 +8544,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:01:41</t>
+          <t>Última actualización: 13:58:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -8885,7 +9535,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8899,7 +9549,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8910,7 +9560,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8924,9 +9574,109 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>102</v>
+        <v>45</v>
       </c>
       <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>15:03</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>65</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>15:08</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>70</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>15:43</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>105</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>15:49</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>111</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8943,7 +9693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8956,14 +9706,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:01:41</t>
+          <t>Última actualización: 13:58:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -9966,6 +10716,81 @@
       <c r="E44" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>14:32</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>34</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>15:12</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>74</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>109</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1769
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E327"/>
+  <dimension ref="A1:E351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:21</t>
+          <t>Última actualización: 14:33:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 322</t>
+          <t>Total filas: 346</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>95</v>
+        <v>40</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4633,7 +4633,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,7 +4748,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -4758,11 +4758,11 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>5</v>
+        <v>65</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5458,11 +5458,11 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5483,11 +5483,11 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_RUTA 36_ESC 70</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6933,11 +6933,11 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6983,7 +6983,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D266" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D267" t="n">
@@ -7023,7 +7023,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -7033,11 +7033,11 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,7 +7048,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -7058,11 +7058,11 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7208,7 +7208,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D275" t="n">
@@ -7483,7 +7483,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D286" t="n">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D287" t="n">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D289" t="n">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7962,7 +7962,7 @@
         </is>
       </c>
       <c r="D305" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,21 +7973,21 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -7998,21 +7998,21 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>14:42</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>101</v>
+        <v>0</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,21 +8048,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>109</v>
+        <v>2</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8073,21 +8073,21 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>53</v>
+        <v>2</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8098,21 +8098,21 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8128,16 +8128,16 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,21 +8148,21 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:42</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>61</v>
+        <v>101</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8173,21 +8173,21 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,21 +8198,21 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>15:03</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>65</v>
+        <v>14</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8223,21 +8223,21 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>15:08</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>70</v>
+        <v>109</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -8248,21 +8248,21 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>15:12</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -8273,21 +8273,21 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>80</v>
+        <v>18</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -8298,21 +8298,21 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>80</v>
+        <v>21</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -8328,16 +8328,16 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>15:21</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>83</v>
+        <v>61</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,21 +8348,21 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8373,21 +8373,21 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>15:33</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>95</v>
+        <v>28</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -8398,21 +8398,21 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>15:37</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>99</v>
+        <v>30</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -8423,21 +8423,21 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>15:43</t>
+          <t>15:08</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>105</v>
+        <v>35</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8448,21 +8448,21 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>106</v>
+        <v>38</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8473,21 +8473,21 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>15:49</t>
+          <t>15:12</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>111</v>
+        <v>39</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8503,18 +8503,618 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D327" t="n">
+        <v>80</v>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D328" t="n">
+        <v>45</v>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>15:21</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D329" t="n">
+        <v>48</v>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D330" t="n">
+        <v>50</v>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D331" t="n">
+        <v>57</v>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>15:33</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D332" t="n">
+        <v>95</v>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>15:36</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D333" t="n">
+        <v>63</v>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>15:37</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D334" t="n">
+        <v>99</v>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>15:42</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D335" t="n">
+        <v>69</v>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>15:43</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D336" t="n">
+        <v>70</v>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>15:43</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D337" t="n">
+        <v>70</v>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D338" t="n">
+        <v>106</v>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
           <t>15:49</t>
         </is>
       </c>
-      <c r="C327" t="inlineStr">
+      <c r="C339" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D327" t="n">
+      <c r="D339" t="n">
+        <v>76</v>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>15:49</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D340" t="n">
+        <v>76</v>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D341" t="n">
+        <v>81</v>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
+        <v>87</v>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>16:01</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D343" t="n">
+        <v>88</v>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D344" t="n">
+        <v>90</v>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>16:06</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D345" t="n">
+        <v>93</v>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D346" t="n">
+        <v>94</v>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>16:13</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D347" t="n">
+        <v>100</v>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>16:18</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D348" t="n">
+        <v>105</v>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>16:21</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D349" t="n">
+        <v>108</v>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D350" t="n">
         <v>111</v>
       </c>
-      <c r="E327" t="inlineStr">
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>11_ESC 3-ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>117</v>
+      </c>
+      <c r="E351" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8544,7 +9144,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:21</t>
+          <t>Última actualización: 14:33:32</t>
         </is>
       </c>
     </row>
@@ -9560,7 +10160,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -9574,7 +10174,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -9585,7 +10185,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -9599,7 +10199,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -9610,7 +10210,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -9624,7 +10224,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -9635,7 +10235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -9649,7 +10249,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -9660,7 +10260,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -9674,7 +10274,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -9693,7 +10293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9706,14 +10306,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:21</t>
+          <t>Última actualización: 14:33:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 42</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -10747,12 +11347,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>15:12</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -10761,7 +11361,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -10772,23 +11372,73 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>15:12</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>39</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>15:47</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>215C_ESC AGRARIA-LA PLATA</t>
         </is>
       </c>
-      <c r="D47" t="n">
+      <c r="D48" t="n">
+        <v>74</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>16:22</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215D_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
         <v>109</v>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1770
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E351"/>
+  <dimension ref="A1:E379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:33:32</t>
+          <t>Última actualización: 15:04:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 346</t>
+          <t>Total filas: 374</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>26</v>
+        <v>76</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1608,11 +1608,11 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>22</v>
+        <v>113</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>113</v>
+        <v>40</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>95</v>
+        <v>40</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4633,7 +4633,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,7 +4748,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -4758,11 +4758,11 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>5</v>
+        <v>65</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5208,11 +5208,11 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6933,11 +6933,11 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_RUTA 36_ESC 70</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,7 +6948,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -6958,11 +6958,11 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>6</v>
+        <v>92</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6983,7 +6983,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D266" t="n">
@@ -6998,7 +6998,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -7008,11 +7008,11 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>92</v>
+        <v>6</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,7 +7023,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -7033,11 +7033,11 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,7 +7048,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -7058,11 +7058,11 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7158,11 +7158,11 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,7 +7173,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -7183,11 +7183,11 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7283,7 +7283,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D278" t="n">
@@ -7308,7 +7308,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D279" t="n">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D289" t="n">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>5</v>
+        <v>62</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7958,7 +7958,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D305" t="n">
@@ -7983,7 +7983,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D306" t="n">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8258,7 +8258,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D317" t="n">
@@ -8283,7 +8283,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D318" t="n">
@@ -8323,7 +8323,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -8333,11 +8333,11 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -8358,11 +8358,11 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8423,21 +8423,21 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>15:08</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8448,21 +8448,21 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8473,21 +8473,21 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>15:12</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8498,21 +8498,21 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8523,21 +8523,21 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8548,21 +8548,21 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>15:21</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8573,21 +8573,21 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -8603,16 +8603,16 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:08</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8623,21 +8623,21 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>15:33</t>
+          <t>15:09</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>95</v>
+        <v>5</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8653,16 +8653,16 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>15:36</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,21 +8673,21 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>15:37</t>
+          <t>15:12</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>99</v>
+        <v>8</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8698,21 +8698,21 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>15:42</t>
+          <t>15:12</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>69</v>
+        <v>8</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,21 +8723,21 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>15:43</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8753,16 +8753,16 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>15:43</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -8773,21 +8773,21 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:19</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>106</v>
+        <v>15</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,21 +8798,21 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>15:49</t>
+          <t>15:21</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8828,16 +8828,16 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>15:49</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -8848,21 +8848,21 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>81</v>
+        <v>20</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8878,16 +8878,16 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -8898,21 +8898,21 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>16:01</t>
+          <t>15:31</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>88</v>
+        <v>27</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -8923,21 +8923,21 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>16:03</t>
+          <t>15:33</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8948,21 +8948,21 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>16:06</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>93</v>
+        <v>30</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8973,21 +8973,21 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>15:36</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>94</v>
+        <v>32</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,21 +8998,21 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>16:13</t>
+          <t>15:37</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9023,21 +9023,21 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>16:18</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>105</v>
+        <v>38</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9053,16 +9053,16 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>15:43</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>108</v>
+        <v>70</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,21 +9073,21 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>15:43</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>111</v>
+        <v>39</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9098,23 +9098,723 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
+          <t>13:58:21</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>106</v>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>15:49</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D352" t="n">
+        <v>45</v>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>15:49</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D353" t="n">
+        <v>45</v>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
           <t>14:33:32</t>
         </is>
       </c>
-      <c r="B351" t="inlineStr">
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D354" t="n">
+        <v>81</v>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D355" t="n">
+        <v>51</v>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>56</v>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>16:01</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D357" t="n">
+        <v>88</v>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>16:02</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D358" t="n">
+        <v>58</v>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D359" t="n">
+        <v>90</v>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D360" t="n">
+        <v>60</v>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>16:06</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D361" t="n">
+        <v>93</v>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D362" t="n">
+        <v>94</v>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>16:13</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D363" t="n">
+        <v>69</v>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D364" t="n">
+        <v>70</v>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>16:18</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D365" t="n">
+        <v>105</v>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>16:19</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D366" t="n">
+        <v>75</v>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>16:21</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D367" t="n">
+        <v>77</v>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D368" t="n">
+        <v>79</v>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D369" t="n">
+        <v>80</v>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>14:33:32</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
         <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="C351" t="inlineStr">
+      <c r="C370" t="inlineStr">
         <is>
           <t>11_ESC 3-ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D351" t="n">
+      <c r="D370" t="n">
         <v>117</v>
       </c>
-      <c r="E351" t="inlineStr">
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>16:31</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>11_ESC 3-ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D371" t="n">
+        <v>87</v>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D372" t="n">
+        <v>94</v>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>16:42</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D373" t="n">
+        <v>98</v>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D374" t="n">
+        <v>102</v>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>16:48</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D375" t="n">
+        <v>104</v>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D376" t="n">
+        <v>109</v>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D377" t="n">
+        <v>111</v>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D378" t="n">
+        <v>112</v>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>16:58</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D379" t="n">
+        <v>114</v>
+      </c>
+      <c r="E379" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9131,7 +9831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9144,14 +9844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:33:32</t>
+          <t>Última actualización: 15:04:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 48</t>
         </is>
       </c>
     </row>
@@ -10210,21 +10910,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>15:08</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -10235,21 +10935,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>15:43</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>70</v>
+        <v>2</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -10265,18 +10965,118 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>15:08</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>35</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>15:43</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>39</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>15:49</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D49" t="n">
-        <v>76</v>
-      </c>
-      <c r="E49" t="inlineStr">
+      <c r="D51" t="n">
+        <v>45</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>109</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>111</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10293,7 +11093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10306,14 +11106,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:33:32</t>
+          <t>Última actualización: 15:04:05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 47</t>
         </is>
       </c>
     </row>
@@ -11397,50 +12197,125 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>74</v>
+        <v>9</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>43</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
           <t>16:22</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>215D_LA PLATA</t>
         </is>
       </c>
-      <c r="D49" t="n">
-        <v>109</v>
-      </c>
-      <c r="E49" t="inlineStr">
+      <c r="D50" t="n">
+        <v>78</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>102</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>16:58</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>114</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1771
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E379"/>
+  <dimension ref="A1:E406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:04:05</t>
+          <t>Última actualización: 16:03:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 374</t>
+          <t>Total filas: 401</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>18</v>
+        <v>86</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>113</v>
+        <v>40</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5208,11 +5208,11 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_RUTA 36_ESC 70</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6908,7 +6908,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6933,11 +6933,11 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D266" t="n">
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7158,11 +7158,11 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7198,7 +7198,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -7208,11 +7208,11 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7483,7 +7483,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D286" t="n">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D287" t="n">
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>5</v>
+        <v>62</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -8258,7 +8258,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D317" t="n">
@@ -8283,7 +8283,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D318" t="n">
@@ -8323,7 +8323,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -8333,11 +8333,11 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -8358,11 +8358,11 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8683,7 +8683,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D334" t="n">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -8723,7 +8723,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -8733,11 +8733,11 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,7 +8748,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
@@ -8758,11 +8758,11 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -9048,7 +9048,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -9058,11 +9058,11 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,7 +9073,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -9083,11 +9083,11 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D352" t="n">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D353" t="n">
@@ -9298,7 +9298,7 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
@@ -9308,11 +9308,11 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -9323,21 +9323,21 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -9348,21 +9348,21 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>16:06</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>93</v>
+        <v>0</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -9378,16 +9378,16 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -9398,21 +9398,21 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>16:13</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
@@ -9423,21 +9423,21 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -9448,21 +9448,21 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>16:18</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>105</v>
+        <v>1</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -9473,21 +9473,21 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>16:19</t>
+          <t>16:06</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>75</v>
+        <v>3</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -9498,21 +9498,21 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:07</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -9523,21 +9523,21 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:13</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -9548,21 +9548,21 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:13</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>11X44-ESC 61_ETCHEVERRY</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D369" t="n">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -9573,21 +9573,21 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>11_ESC 3-ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>117</v>
+        <v>70</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -9598,21 +9598,21 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>16:31</t>
+          <t>16:18</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>11_ESC 3-ETCHEVERRY</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>87</v>
+        <v>15</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -9628,16 +9628,16 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:19</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D372" t="n">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="E372" t="inlineStr">
         <is>
@@ -9648,21 +9648,21 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>16:42</t>
+          <t>16:21</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>98</v>
+        <v>18</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -9673,21 +9673,21 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>16:46</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>102</v>
+        <v>20</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -9698,21 +9698,21 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>16:48</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>104</v>
+        <v>20</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -9723,21 +9723,21 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>16:53</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44-ESC 61_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>109</v>
+        <v>21</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -9748,21 +9748,21 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>11_ESC 3-ETCHEVERRY</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>111</v>
+        <v>27</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -9778,16 +9778,16 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:31</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>11_ESC 3-ETCHEVERRY</t>
         </is>
       </c>
       <c r="D378" t="n">
-        <v>112</v>
+        <v>87</v>
       </c>
       <c r="E378" t="inlineStr">
         <is>
@@ -9803,18 +9803,693 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D379" t="n">
+        <v>94</v>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D380" t="n">
+        <v>38</v>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>16:42</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D381" t="n">
+        <v>98</v>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D382" t="n">
+        <v>42</v>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D383" t="n">
+        <v>43</v>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>16:47</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D384" t="n">
+        <v>44</v>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>16:48</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D385" t="n">
+        <v>45</v>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>16:48</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D386" t="n">
+        <v>104</v>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>16:52</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D387" t="n">
+        <v>49</v>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D388" t="n">
+        <v>109</v>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-EL PATO</t>
+        </is>
+      </c>
+      <c r="D389" t="n">
+        <v>52</v>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D390" t="n">
+        <v>53</v>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
           <t>16:58</t>
         </is>
       </c>
-      <c r="C379" t="inlineStr">
+      <c r="C391" t="inlineStr">
         <is>
           <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
-      <c r="D379" t="n">
-        <v>114</v>
-      </c>
-      <c r="E379" t="inlineStr">
+      <c r="D391" t="n">
+        <v>55</v>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D392" t="n">
+        <v>57</v>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>17:01</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D393" t="n">
+        <v>58</v>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>17:05</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D394" t="n">
+        <v>62</v>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>17:07</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D395" t="n">
+        <v>64</v>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D396" t="n">
+        <v>67</v>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D397" t="n">
+        <v>71</v>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D398" t="n">
+        <v>72</v>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D399" t="n">
+        <v>79</v>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D400" t="n">
+        <v>92</v>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D401" t="n">
+        <v>92</v>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>17:43</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D402" t="n">
+        <v>100</v>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D403" t="n">
+        <v>112</v>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D404" t="n">
+        <v>116</v>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D405" t="n">
+        <v>116</v>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D406" t="n">
+        <v>117</v>
+      </c>
+      <c r="E406" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9831,7 +10506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9844,14 +10519,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:04:05</t>
+          <t>Última actualización: 16:03:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 48</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -11035,12 +11710,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>16:53</t>
+          <t>16:52</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -11049,7 +11724,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>109</v>
+        <v>49</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -11065,18 +11740,68 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>109</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
           <t>16:55</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
-      <c r="D53" t="n">
-        <v>111</v>
-      </c>
-      <c r="E53" t="inlineStr">
+      <c r="D54" t="n">
+        <v>52</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>72</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11093,7 +11818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11106,14 +11831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:04:05</t>
+          <t>Última actualización: 16:03:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 47</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -12247,7 +12972,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -12261,7 +12986,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -12272,12 +12997,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>16:46</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -12286,7 +13011,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>102</v>
+        <v>42</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -12302,20 +13027,95 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>102</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>16:57</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>54</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>15:04:05</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
           <t>16:58</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D52" t="n">
+      <c r="D54" t="n">
         <v>114</v>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>17:25</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>82</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1772
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E406"/>
+  <dimension ref="A1:E426"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:03:30</t>
+          <t>Última actualización: 16:42:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 401</t>
+          <t>Total filas: 421</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -658,11 +658,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -683,11 +683,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>95</v>
+        <v>40</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4633,7 +4633,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5208,11 +5208,11 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5458,11 +5458,11 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5483,11 +5483,11 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D223" t="n">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6948,7 +6948,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -6958,11 +6958,11 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>92</v>
+        <v>6</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6983,7 +6983,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D266" t="n">
@@ -6998,7 +6998,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -7008,11 +7008,11 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>6</v>
+        <v>92</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7158,11 +7158,11 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7198,7 +7198,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -7208,11 +7208,11 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7483,7 +7483,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D286" t="n">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D287" t="n">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D305" t="n">
@@ -7983,7 +7983,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D306" t="n">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8258,7 +8258,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D317" t="n">
@@ -8283,7 +8283,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D318" t="n">
@@ -8323,7 +8323,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -8333,11 +8333,11 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -8358,11 +8358,11 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8433,7 +8433,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D324" t="n">
@@ -8458,7 +8458,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D325" t="n">
@@ -9048,7 +9048,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -9058,11 +9058,11 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,7 +9073,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -9083,11 +9083,11 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D352" t="n">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D353" t="n">
@@ -9308,7 +9308,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D359" t="n">
@@ -9323,7 +9323,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
@@ -9333,11 +9333,11 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -9373,7 +9373,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -9383,11 +9383,11 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -9408,7 +9408,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D363" t="n">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D365" t="n">
@@ -9533,7 +9533,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D368" t="n">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D369" t="n">
@@ -9873,12 +9873,12 @@
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>16:45</t>
+          <t>16:43</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
@@ -9887,7 +9887,7 @@
         </is>
       </c>
       <c r="D382" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E382" t="inlineStr">
         <is>
@@ -9898,21 +9898,21 @@
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>16:46</t>
+          <t>16:43</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D383" t="n">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="E383" t="inlineStr">
         <is>
@@ -9923,21 +9923,21 @@
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>44</v>
+        <v>3</v>
       </c>
       <c r="E384" t="inlineStr">
         <is>
@@ -9953,16 +9953,16 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>16:48</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E385" t="inlineStr">
         <is>
@@ -9973,21 +9973,21 @@
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>16:48</t>
+          <t>16:46</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D386" t="n">
-        <v>104</v>
+        <v>4</v>
       </c>
       <c r="E386" t="inlineStr">
         <is>
@@ -9998,21 +9998,21 @@
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>16:52</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D387" t="n">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="E387" t="inlineStr">
         <is>
@@ -10028,16 +10028,16 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>16:53</t>
+          <t>16:48</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="E388" t="inlineStr">
         <is>
@@ -10053,16 +10053,16 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:48</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>215C_ESC AGRARIA-EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="E389" t="inlineStr">
         <is>
@@ -10073,21 +10073,21 @@
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:52</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D390" t="n">
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="E390" t="inlineStr">
         <is>
@@ -10098,21 +10098,21 @@
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>16:58</t>
+          <t>16:52</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D391" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="E391" t="inlineStr">
         <is>
@@ -10123,21 +10123,21 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:53</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>57</v>
+        <v>109</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -10148,21 +10148,21 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>16:53</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>58</v>
+        <v>11</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -10173,21 +10173,21 @@
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_ESC AGRARIA-EL PATO</t>
         </is>
       </c>
       <c r="D394" t="n">
-        <v>62</v>
+        <v>13</v>
       </c>
       <c r="E394" t="inlineStr">
         <is>
@@ -10198,21 +10198,21 @@
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D395" t="n">
-        <v>64</v>
+        <v>14</v>
       </c>
       <c r="E395" t="inlineStr">
         <is>
@@ -10228,16 +10228,16 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>16:58</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D396" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="E396" t="inlineStr">
         <is>
@@ -10253,16 +10253,16 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D397" t="n">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="E397" t="inlineStr">
         <is>
@@ -10273,21 +10273,21 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>72</v>
+        <v>19</v>
       </c>
       <c r="E398" t="inlineStr">
         <is>
@@ -10298,21 +10298,21 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D399" t="n">
-        <v>79</v>
+        <v>23</v>
       </c>
       <c r="E399" t="inlineStr">
         <is>
@@ -10323,21 +10323,21 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D400" t="n">
-        <v>92</v>
+        <v>25</v>
       </c>
       <c r="E400" t="inlineStr">
         <is>
@@ -10348,21 +10348,21 @@
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D401" t="n">
-        <v>92</v>
+        <v>28</v>
       </c>
       <c r="E401" t="inlineStr">
         <is>
@@ -10373,21 +10373,21 @@
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>17:43</t>
+          <t>17:13</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D402" t="n">
-        <v>100</v>
+        <v>31</v>
       </c>
       <c r="E402" t="inlineStr">
         <is>
@@ -10403,16 +10403,16 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D403" t="n">
-        <v>112</v>
+        <v>71</v>
       </c>
       <c r="E403" t="inlineStr">
         <is>
@@ -10423,21 +10423,21 @@
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D404" t="n">
-        <v>116</v>
+        <v>33</v>
       </c>
       <c r="E404" t="inlineStr">
         <is>
@@ -10448,21 +10448,21 @@
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D405" t="n">
-        <v>116</v>
+        <v>33</v>
       </c>
       <c r="E405" t="inlineStr">
         <is>
@@ -10473,23 +10473,523 @@
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D406" t="n">
+        <v>33</v>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D407" t="n">
+        <v>39</v>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
           <t>16:03:30</t>
         </is>
       </c>
-      <c r="B406" t="inlineStr">
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D408" t="n">
+        <v>79</v>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D409" t="n">
+        <v>48</v>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D410" t="n">
+        <v>53</v>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D411" t="n">
+        <v>53</v>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D412" t="n">
+        <v>58</v>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>17:43</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D413" t="n">
+        <v>61</v>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>17:51</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D414" t="n">
+        <v>69</v>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D415" t="n">
+        <v>112</v>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>17:56</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D416" t="n">
+        <v>74</v>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D417" t="n">
+        <v>116</v>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D418" t="n">
+        <v>77</v>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
         <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="C406" t="inlineStr">
+      <c r="C419" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D406" t="n">
-        <v>117</v>
-      </c>
-      <c r="E406" t="inlineStr">
+      <c r="D419" t="n">
+        <v>78</v>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D420" t="n">
+        <v>78</v>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D421" t="n">
+        <v>83</v>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>18:17</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D422" t="n">
+        <v>95</v>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>18:21</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D423" t="n">
+        <v>99</v>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D424" t="n">
+        <v>108</v>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D425" t="n">
+        <v>115</v>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>18:40</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D426" t="n">
+        <v>118</v>
+      </c>
+      <c r="E426" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10506,7 +11006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10519,14 +11019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:03:30</t>
+          <t>Última actualización: 16:42:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 50</t>
+          <t>Total filas: 51</t>
         </is>
       </c>
     </row>
@@ -11710,7 +12210,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -11724,7 +12224,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -11760,7 +12260,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -11774,7 +12274,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -11785,7 +12285,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -11799,9 +12299,34 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>115</v>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11818,7 +12343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11831,14 +12356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:03:30</t>
+          <t>Última actualización: 16:42:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 50</t>
+          <t>Total filas: 54</t>
         </is>
       </c>
     </row>
@@ -12997,12 +13522,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>16:45</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -13011,7 +13536,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>42</v>
+        <v>2</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -13022,12 +13547,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>16:46</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -13036,7 +13561,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>102</v>
+        <v>42</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -13047,21 +13572,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>16:57</t>
+          <t>16:46</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>54</v>
+        <v>102</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -13072,12 +13597,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>16:58</t>
+          <t>16:57</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -13086,7 +13611,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>114</v>
+        <v>15</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -13097,23 +13622,123 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>16:58</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>114</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>17:25</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D55" t="n">
-        <v>82</v>
-      </c>
-      <c r="E55" t="inlineStr">
+      <c r="D56" t="n">
+        <v>43</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>83</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>101</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>109</v>
+      </c>
+      <c r="E59" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1773
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E426"/>
+  <dimension ref="A1:E449"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:42:24</t>
+          <t>Última actualización: 17:01:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 421</t>
+          <t>Total filas: 444</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -658,11 +658,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -683,11 +683,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4248,7 +4248,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4258,11 +4258,11 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4633,7 +4633,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4858,7 +4858,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5458,11 +5458,11 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5483,11 +5483,11 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6933,11 +6933,11 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_RUTA 36_ESC 70</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -7023,7 +7023,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -7033,11 +7033,11 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,7 +7048,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -7058,11 +7058,11 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7158,11 +7158,11 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7198,7 +7198,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -7208,11 +7208,11 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>5</v>
+        <v>62</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7958,7 +7958,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D305" t="n">
@@ -7983,7 +7983,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D306" t="n">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8258,7 +8258,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D317" t="n">
@@ -8283,7 +8283,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D318" t="n">
@@ -8323,7 +8323,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -8333,11 +8333,11 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -8358,11 +8358,11 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8508,7 +8508,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D327" t="n">
@@ -8533,7 +8533,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D328" t="n">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D330" t="n">
@@ -8723,7 +8723,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -8733,11 +8733,11 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,7 +8748,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
@@ -8758,11 +8758,11 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -9323,7 +9323,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
@@ -9333,11 +9333,11 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -9358,7 +9358,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -9373,7 +9373,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -9383,11 +9383,11 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -9408,7 +9408,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D363" t="n">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D365" t="n">
@@ -9533,7 +9533,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D368" t="n">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D369" t="n">
@@ -9683,7 +9683,7 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D374" t="n">
@@ -9708,7 +9708,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D375" t="n">
@@ -9883,7 +9883,7 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D382" t="n">
@@ -9908,7 +9908,7 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D383" t="n">
@@ -10023,7 +10023,7 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
@@ -10033,11 +10033,11 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>104</v>
+        <v>45</v>
       </c>
       <c r="E388" t="inlineStr">
         <is>
@@ -10048,7 +10048,7 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
@@ -10058,11 +10058,11 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>45</v>
+        <v>104</v>
       </c>
       <c r="E389" t="inlineStr">
         <is>
@@ -10083,7 +10083,7 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D390" t="n">
@@ -10108,7 +10108,7 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D391" t="n">
@@ -10298,21 +10298,21 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D399" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E399" t="inlineStr">
         <is>
@@ -10323,21 +10323,21 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D400" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E400" t="inlineStr">
         <is>
@@ -10348,21 +10348,21 @@
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>17:02</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D401" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E401" t="inlineStr">
         <is>
@@ -10373,21 +10373,21 @@
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>17:13</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D402" t="n">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="E402" t="inlineStr">
         <is>
@@ -10398,21 +10398,21 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D403" t="n">
-        <v>71</v>
+        <v>4</v>
       </c>
       <c r="E403" t="inlineStr">
         <is>
@@ -10428,16 +10428,16 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D404" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="E404" t="inlineStr">
         <is>
@@ -10448,21 +10448,21 @@
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D405" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E405" t="inlineStr">
         <is>
@@ -10473,21 +10473,21 @@
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D406" t="n">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="E406" t="inlineStr">
         <is>
@@ -10498,21 +10498,21 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:13</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D407" t="n">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="E407" t="inlineStr">
         <is>
@@ -10523,21 +10523,21 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D408" t="n">
-        <v>79</v>
+        <v>13</v>
       </c>
       <c r="E408" t="inlineStr">
         <is>
@@ -10548,21 +10548,21 @@
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D409" t="n">
-        <v>48</v>
+        <v>13</v>
       </c>
       <c r="E409" t="inlineStr">
         <is>
@@ -10578,16 +10578,16 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D410" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="E410" t="inlineStr">
         <is>
@@ -10603,16 +10603,16 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D411" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="E411" t="inlineStr">
         <is>
@@ -10628,16 +10628,16 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D412" t="n">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="E412" t="inlineStr">
         <is>
@@ -10648,21 +10648,21 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>17:43</t>
+          <t>17:20</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D413" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="E413" t="inlineStr">
         <is>
@@ -10673,21 +10673,21 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:20</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D414" t="n">
-        <v>69</v>
+        <v>19</v>
       </c>
       <c r="E414" t="inlineStr">
         <is>
@@ -10698,21 +10698,21 @@
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D415" t="n">
-        <v>112</v>
+        <v>39</v>
       </c>
       <c r="E415" t="inlineStr">
         <is>
@@ -10723,21 +10723,21 @@
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>17:56</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D416" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E416" t="inlineStr">
         <is>
@@ -10748,21 +10748,21 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D417" t="n">
-        <v>116</v>
+        <v>29</v>
       </c>
       <c r="E417" t="inlineStr">
         <is>
@@ -10773,21 +10773,21 @@
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:34</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D418" t="n">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="E418" t="inlineStr">
         <is>
@@ -10803,16 +10803,16 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D419" t="n">
-        <v>78</v>
+        <v>53</v>
       </c>
       <c r="E419" t="inlineStr">
         <is>
@@ -10823,21 +10823,21 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D420" t="n">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="E420" t="inlineStr">
         <is>
@@ -10848,21 +10848,21 @@
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D421" t="n">
-        <v>83</v>
+        <v>37</v>
       </c>
       <c r="E421" t="inlineStr">
         <is>
@@ -10873,21 +10873,21 @@
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>18:17</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D422" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="E422" t="inlineStr">
         <is>
@@ -10898,21 +10898,21 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>17:42</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D423" t="n">
-        <v>99</v>
+        <v>41</v>
       </c>
       <c r="E423" t="inlineStr">
         <is>
@@ -10928,16 +10928,16 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>17:43</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D424" t="n">
-        <v>108</v>
+        <v>61</v>
       </c>
       <c r="E424" t="inlineStr">
         <is>
@@ -10953,16 +10953,16 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>17:51</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D425" t="n">
-        <v>115</v>
+        <v>69</v>
       </c>
       <c r="E425" t="inlineStr">
         <is>
@@ -10973,23 +10973,598 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D426" t="n">
+        <v>54</v>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D427" t="n">
+        <v>112</v>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
           <t>16:42:24</t>
         </is>
       </c>
-      <c r="B426" t="inlineStr">
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>17:56</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D428" t="n">
+        <v>74</v>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>17:57</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D429" t="n">
+        <v>56</v>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D430" t="n">
+        <v>58</v>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D431" t="n">
+        <v>58</v>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>16:03:30</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D432" t="n">
+        <v>116</v>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D433" t="n">
+        <v>78</v>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D434" t="n">
+        <v>78</v>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D435" t="n">
+        <v>63</v>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D436" t="n">
+        <v>83</v>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>18:07</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D437" t="n">
+        <v>66</v>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>18:07</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D438" t="n">
+        <v>66</v>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>18:17</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D439" t="n">
+        <v>95</v>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D440" t="n">
+        <v>79</v>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D441" t="n">
+        <v>79</v>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>18:21</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D442" t="n">
+        <v>99</v>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D443" t="n">
+        <v>108</v>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D444" t="n">
+        <v>95</v>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D445" t="n">
+        <v>115</v>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
         <is>
           <t>18:40</t>
         </is>
       </c>
-      <c r="C426" t="inlineStr">
+      <c r="C446" t="inlineStr">
         <is>
           <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
-      <c r="D426" t="n">
-        <v>118</v>
-      </c>
-      <c r="E426" t="inlineStr">
+      <c r="D446" t="n">
+        <v>99</v>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D447" t="n">
+        <v>101</v>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D448" t="n">
+        <v>101</v>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>18:49</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D449" t="n">
+        <v>108</v>
+      </c>
+      <c r="E449" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11006,7 +11581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11019,14 +11594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:42:24</t>
+          <t>Última actualización: 17:01:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 51</t>
+          <t>Total filas: 55</t>
         </is>
       </c>
     </row>
@@ -12285,12 +12860,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -12299,7 +12874,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -12315,18 +12890,118 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>33</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>95</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
           <t>18:37</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D56" t="n">
+      <c r="D58" t="n">
         <v>115</v>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>101</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>101</v>
+      </c>
+      <c r="E60" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -12343,7 +13018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12356,14 +13031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:42:24</t>
+          <t>Última actualización: 17:01:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 54</t>
+          <t>Total filas: 57</t>
         </is>
       </c>
     </row>
@@ -13647,12 +14322,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>17:25</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -13661,7 +14336,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -13677,41 +14352,41 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>101</v>
+        <v>64</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -13722,25 +14397,100 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>82</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>89</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>16:42:24</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>18:31</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D59" t="n">
+      <c r="D61" t="n">
         <v>109</v>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>109</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1774
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E449"/>
+  <dimension ref="A1:E469"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:01:59</t>
+          <t>Última actualización: 17:47:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 444</t>
+          <t>Total filas: 464</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1608,11 +1608,11 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>26</v>
+        <v>76</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>22</v>
+        <v>113</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4248,7 +4248,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4258,11 +4258,11 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4858,7 +4858,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6948,7 +6948,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -6958,11 +6958,11 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>6</v>
+        <v>92</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6983,7 +6983,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D266" t="n">
@@ -6998,7 +6998,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -7008,11 +7008,11 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>92</v>
+        <v>6</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,7 +7023,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -7033,11 +7033,11 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,7 +7048,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -7058,11 +7058,11 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7483,7 +7483,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D286" t="n">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D287" t="n">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D289" t="n">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>5</v>
+        <v>62</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7958,7 +7958,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D305" t="n">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8258,7 +8258,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D317" t="n">
@@ -8283,7 +8283,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D318" t="n">
@@ -8323,7 +8323,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -8333,11 +8333,11 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -8358,11 +8358,11 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8483,7 +8483,7 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D326" t="n">
@@ -8533,7 +8533,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D328" t="n">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D330" t="n">
@@ -8683,7 +8683,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D334" t="n">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -9048,7 +9048,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -9058,11 +9058,11 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,7 +9073,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -9083,11 +9083,11 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D352" t="n">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D353" t="n">
@@ -9308,7 +9308,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D359" t="n">
@@ -9333,7 +9333,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D360" t="n">
@@ -9358,7 +9358,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -9408,7 +9408,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D363" t="n">
@@ -9433,7 +9433,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D364" t="n">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D365" t="n">
@@ -9883,7 +9883,7 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D382" t="n">
@@ -9908,7 +9908,7 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D383" t="n">
@@ -9923,7 +9923,7 @@
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
@@ -9933,11 +9933,11 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="E384" t="inlineStr">
         <is>
@@ -9948,7 +9948,7 @@
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
@@ -9958,11 +9958,11 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="E385" t="inlineStr">
         <is>
@@ -10023,7 +10023,7 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
@@ -10033,11 +10033,11 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>45</v>
+        <v>104</v>
       </c>
       <c r="E388" t="inlineStr">
         <is>
@@ -10048,7 +10048,7 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
@@ -10058,11 +10058,11 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>104</v>
+        <v>45</v>
       </c>
       <c r="E389" t="inlineStr">
         <is>
@@ -10273,7 +10273,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
@@ -10283,11 +10283,11 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E398" t="inlineStr">
         <is>
@@ -10308,7 +10308,7 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D399" t="n">
@@ -10323,7 +10323,7 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
@@ -10333,11 +10333,11 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D400" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E400" t="inlineStr">
         <is>
@@ -10533,7 +10533,7 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D408" t="n">
@@ -10558,7 +10558,7 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D409" t="n">
@@ -10583,7 +10583,7 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D410" t="n">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D411" t="n">
@@ -10633,7 +10633,7 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D412" t="n">
@@ -10948,21 +10948,21 @@
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D425" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="E425" t="inlineStr">
         <is>
@@ -10973,21 +10973,21 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D426" t="n">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="E426" t="inlineStr">
         <is>
@@ -10998,21 +10998,21 @@
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:48</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D427" t="n">
-        <v>112</v>
+        <v>1</v>
       </c>
       <c r="E427" t="inlineStr">
         <is>
@@ -11023,21 +11023,21 @@
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>17:56</t>
+          <t>17:48</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D428" t="n">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="E428" t="inlineStr">
         <is>
@@ -11048,21 +11048,21 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>17:57</t>
+          <t>17:51</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D429" t="n">
-        <v>56</v>
+        <v>4</v>
       </c>
       <c r="E429" t="inlineStr">
         <is>
@@ -11073,21 +11073,21 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:51</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D430" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E430" t="inlineStr">
         <is>
@@ -11103,16 +11103,16 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D431" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E431" t="inlineStr">
         <is>
@@ -11128,16 +11128,16 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D432" t="n">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E432" t="inlineStr">
         <is>
@@ -11153,16 +11153,16 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:56</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D433" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="E433" t="inlineStr">
         <is>
@@ -11173,21 +11173,21 @@
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:57</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D434" t="n">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="E434" t="inlineStr">
         <is>
@@ -11203,16 +11203,16 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D435" t="n">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="E435" t="inlineStr">
         <is>
@@ -11223,21 +11223,21 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D436" t="n">
-        <v>83</v>
+        <v>116</v>
       </c>
       <c r="E436" t="inlineStr">
         <is>
@@ -11248,21 +11248,21 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>18:07</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D437" t="n">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="E437" t="inlineStr">
         <is>
@@ -11273,21 +11273,21 @@
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>18:07</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D438" t="n">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="E438" t="inlineStr">
         <is>
@@ -11303,16 +11303,16 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>18:17</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D439" t="n">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="E439" t="inlineStr">
         <is>
@@ -11323,21 +11323,21 @@
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:02</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D440" t="n">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="E440" t="inlineStr">
         <is>
@@ -11348,21 +11348,21 @@
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D441" t="n">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="E441" t="inlineStr">
         <is>
@@ -11378,16 +11378,16 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D442" t="n">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="E442" t="inlineStr">
         <is>
@@ -11398,21 +11398,21 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:06</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D443" t="n">
-        <v>108</v>
+        <v>19</v>
       </c>
       <c r="E443" t="inlineStr">
         <is>
@@ -11428,16 +11428,16 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:07</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D444" t="n">
-        <v>95</v>
+        <v>66</v>
       </c>
       <c r="E444" t="inlineStr">
         <is>
@@ -11448,21 +11448,21 @@
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:07</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D445" t="n">
-        <v>115</v>
+        <v>20</v>
       </c>
       <c r="E445" t="inlineStr">
         <is>
@@ -11473,21 +11473,21 @@
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>18:40</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D446" t="n">
-        <v>99</v>
+        <v>27</v>
       </c>
       <c r="E446" t="inlineStr">
         <is>
@@ -11498,21 +11498,21 @@
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>18:42</t>
+          <t>18:17</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D447" t="n">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E447" t="inlineStr">
         <is>
@@ -11523,21 +11523,21 @@
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>18:42</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D448" t="n">
-        <v>101</v>
+        <v>33</v>
       </c>
       <c r="E448" t="inlineStr">
         <is>
@@ -11553,18 +11553,518 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D449" t="n">
+        <v>79</v>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D450" t="n">
+        <v>79</v>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>18:21</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D451" t="n">
+        <v>34</v>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D452" t="n">
+        <v>38</v>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>16:42:24</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D453" t="n">
+        <v>108</v>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D454" t="n">
+        <v>47</v>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D455" t="n">
+        <v>95</v>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D456" t="n">
+        <v>50</v>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>18:40</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D457" t="n">
+        <v>53</v>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D458" t="n">
+        <v>55</v>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D459" t="n">
+        <v>55</v>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>17:01:59</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
           <t>18:49</t>
         </is>
       </c>
-      <c r="C449" t="inlineStr">
+      <c r="C460" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D449" t="n">
+      <c r="D460" t="n">
         <v>108</v>
       </c>
-      <c r="E449" t="inlineStr">
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D461" t="n">
+        <v>63</v>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>19:07</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D462" t="n">
+        <v>80</v>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>19:11</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D463" t="n">
+        <v>84</v>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D464" t="n">
+        <v>90</v>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>19:19</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D465" t="n">
+        <v>92</v>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D466" t="n">
+        <v>94</v>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D467" t="n">
+        <v>96</v>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D468" t="n">
+        <v>97</v>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>19:28</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D469" t="n">
+        <v>101</v>
+      </c>
+      <c r="E469" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11581,7 +12081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11594,14 +12094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:01:59</t>
+          <t>Última actualización: 17:47:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 55</t>
+          <t>Total filas: 56</t>
         </is>
       </c>
     </row>
@@ -12935,7 +13435,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -12949,7 +13449,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -12960,7 +13460,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -12974,7 +13474,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>101</v>
+        <v>55</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -12985,7 +13485,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -12999,9 +13499,34 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>101</v>
+        <v>55</v>
       </c>
       <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>90</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -13018,7 +13543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13031,14 +13556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:01:59</t>
+          <t>Última actualización: 17:47:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 57</t>
+          <t>Total filas: 59</t>
         </is>
       </c>
     </row>
@@ -14372,7 +14897,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -14386,7 +14911,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -14422,37 +14947,37 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:29</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>89</v>
+        <v>42</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>18:31</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -14461,7 +14986,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>109</v>
+        <v>89</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -14472,23 +14997,73 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>18:31</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D62" t="n">
         <v>109</v>
       </c>
       <c r="E62" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>18:39</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>52</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>63</v>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1775
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E469"/>
+  <dimension ref="A1:E488"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:47:44</t>
+          <t>Última actualización: 18:15:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 464</t>
+          <t>Total filas: 483</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>26</v>
+        <v>76</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1608,11 +1608,11 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_RUTA 36_ESC 70</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6933,11 +6933,11 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -7958,7 +7958,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D305" t="n">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8258,7 +8258,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D317" t="n">
@@ -8283,7 +8283,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D318" t="n">
@@ -8323,7 +8323,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -8333,11 +8333,11 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -8358,11 +8358,11 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8483,7 +8483,7 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D326" t="n">
@@ -8508,7 +8508,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D327" t="n">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D330" t="n">
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D352" t="n">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D353" t="n">
@@ -9308,7 +9308,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D359" t="n">
@@ -9323,7 +9323,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
@@ -9333,11 +9333,11 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -9358,7 +9358,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -9373,7 +9373,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -9383,11 +9383,11 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -9408,7 +9408,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D363" t="n">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D365" t="n">
@@ -9683,7 +9683,7 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D374" t="n">
@@ -9708,7 +9708,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D375" t="n">
@@ -10123,7 +10123,7 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
@@ -10133,11 +10133,11 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>109</v>
+        <v>11</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -10148,7 +10148,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
@@ -10158,11 +10158,11 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>11</v>
+        <v>109</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -10298,7 +10298,7 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
@@ -10308,11 +10308,11 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D399" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E399" t="inlineStr">
         <is>
@@ -10323,7 +10323,7 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
@@ -10333,11 +10333,11 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D400" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E400" t="inlineStr">
         <is>
@@ -10533,7 +10533,7 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D408" t="n">
@@ -10558,7 +10558,7 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D409" t="n">
@@ -10658,7 +10658,7 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D413" t="n">
@@ -10683,7 +10683,7 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D414" t="n">
@@ -10958,7 +10958,7 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D425" t="n">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D426" t="n">
@@ -11048,7 +11048,7 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
@@ -11058,11 +11058,11 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D429" t="n">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="E429" t="inlineStr">
         <is>
@@ -11073,7 +11073,7 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
@@ -11083,11 +11083,11 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D430" t="n">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="E430" t="inlineStr">
         <is>
@@ -11098,7 +11098,7 @@
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
@@ -11108,11 +11108,11 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D431" t="n">
-        <v>54</v>
+        <v>112</v>
       </c>
       <c r="E431" t="inlineStr">
         <is>
@@ -11123,7 +11123,7 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
@@ -11133,11 +11133,11 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D432" t="n">
-        <v>112</v>
+        <v>54</v>
       </c>
       <c r="E432" t="inlineStr">
         <is>
@@ -11198,7 +11198,7 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
@@ -11208,11 +11208,11 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D435" t="n">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="E435" t="inlineStr">
         <is>
@@ -11223,7 +11223,7 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
@@ -11233,11 +11233,11 @@
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D436" t="n">
-        <v>116</v>
+        <v>58</v>
       </c>
       <c r="E436" t="inlineStr">
         <is>
@@ -11248,7 +11248,7 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
@@ -11258,11 +11258,11 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D437" t="n">
-        <v>12</v>
+        <v>116</v>
       </c>
       <c r="E437" t="inlineStr">
         <is>
@@ -11283,7 +11283,7 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D438" t="n">
@@ -11308,7 +11308,7 @@
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D439" t="n">
@@ -11498,21 +11498,21 @@
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>18:17</t>
+          <t>18:16</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D447" t="n">
-        <v>95</v>
+        <v>1</v>
       </c>
       <c r="E447" t="inlineStr">
         <is>
@@ -11523,21 +11523,21 @@
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:17</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D448" t="n">
-        <v>33</v>
+        <v>95</v>
       </c>
       <c r="E448" t="inlineStr">
         <is>
@@ -11548,7 +11548,7 @@
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
@@ -11558,11 +11558,11 @@
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D449" t="n">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="E449" t="inlineStr">
         <is>
@@ -11598,21 +11598,21 @@
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D451" t="n">
-        <v>34</v>
+        <v>79</v>
       </c>
       <c r="E451" t="inlineStr">
         <is>
@@ -11623,21 +11623,21 @@
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D452" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="E452" t="inlineStr">
         <is>
@@ -11648,21 +11648,21 @@
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D453" t="n">
-        <v>108</v>
+        <v>6</v>
       </c>
       <c r="E453" t="inlineStr">
         <is>
@@ -11673,21 +11673,21 @@
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D454" t="n">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="E454" t="inlineStr">
         <is>
@@ -11698,21 +11698,21 @@
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D455" t="n">
-        <v>95</v>
+        <v>10</v>
       </c>
       <c r="E455" t="inlineStr">
         <is>
@@ -11723,21 +11723,21 @@
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:28</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D456" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E456" t="inlineStr">
         <is>
@@ -11748,21 +11748,21 @@
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>18:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D457" t="n">
-        <v>53</v>
+        <v>108</v>
       </c>
       <c r="E457" t="inlineStr">
         <is>
@@ -11773,21 +11773,21 @@
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>18:42</t>
+          <t>18:31</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D458" t="n">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="E458" t="inlineStr">
         <is>
@@ -11803,16 +11803,16 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>18:42</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D459" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E459" t="inlineStr">
         <is>
@@ -11828,16 +11828,16 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>18:49</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D460" t="n">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="E460" t="inlineStr">
         <is>
@@ -11848,21 +11848,21 @@
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D461" t="n">
-        <v>63</v>
+        <v>22</v>
       </c>
       <c r="E461" t="inlineStr">
         <is>
@@ -11873,21 +11873,21 @@
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>19:07</t>
+          <t>18:40</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D462" t="n">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="E462" t="inlineStr">
         <is>
@@ -11898,21 +11898,21 @@
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>18:42</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D463" t="n">
-        <v>84</v>
+        <v>27</v>
       </c>
       <c r="E463" t="inlineStr">
         <is>
@@ -11928,16 +11928,16 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>18:42</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D464" t="n">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="E464" t="inlineStr">
         <is>
@@ -11948,21 +11948,21 @@
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>18:43</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D465" t="n">
-        <v>92</v>
+        <v>28</v>
       </c>
       <c r="E465" t="inlineStr">
         <is>
@@ -11973,21 +11973,21 @@
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>18:45</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D466" t="n">
-        <v>94</v>
+        <v>30</v>
       </c>
       <c r="E466" t="inlineStr">
         <is>
@@ -11998,21 +11998,21 @@
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>18:49</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D467" t="n">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="E467" t="inlineStr">
         <is>
@@ -12028,16 +12028,16 @@
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>18:50</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D468" t="n">
-        <v>97</v>
+        <v>63</v>
       </c>
       <c r="E468" t="inlineStr">
         <is>
@@ -12048,23 +12048,498 @@
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D469" t="n">
+        <v>38</v>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D470" t="n">
+        <v>40</v>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
           <t>17:47:44</t>
         </is>
       </c>
-      <c r="B469" t="inlineStr">
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>19:07</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D471" t="n">
+        <v>80</v>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D472" t="n">
+        <v>53</v>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>19:11</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D473" t="n">
+        <v>84</v>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>19:12</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D474" t="n">
+        <v>57</v>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D475" t="n">
+        <v>62</v>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D476" t="n">
+        <v>63</v>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>19:19</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D477" t="n">
+        <v>64</v>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>19:19</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D478" t="n">
+        <v>64</v>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D479" t="n">
+        <v>94</v>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D480" t="n">
+        <v>96</v>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D481" t="n">
+        <v>97</v>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
         <is>
           <t>19:28</t>
         </is>
       </c>
-      <c r="C469" t="inlineStr">
+      <c r="C482" t="inlineStr">
         <is>
           <t>26_HERNANDEZ</t>
         </is>
       </c>
-      <c r="D469" t="n">
+      <c r="D482" t="n">
         <v>101</v>
       </c>
-      <c r="E469" t="inlineStr">
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D483" t="n">
+        <v>81</v>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D484" t="n">
+        <v>88</v>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>19:48</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D485" t="n">
+        <v>93</v>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>19:51</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D486" t="n">
+        <v>96</v>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>19:52</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D487" t="n">
+        <v>97</v>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>19:58</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D488" t="n">
+        <v>103</v>
+      </c>
+      <c r="E488" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -12081,7 +12556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12094,14 +12569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:47:44</t>
+          <t>Última actualización: 18:15:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 56</t>
+          <t>Total filas: 57</t>
         </is>
       </c>
     </row>
@@ -13435,7 +13910,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -13449,7 +13924,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -13485,7 +13960,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -13499,7 +13974,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -13510,23 +13985,48 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
+          <t>18:43</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>28</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
           <t>19:17</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D61" t="n">
-        <v>90</v>
-      </c>
-      <c r="E61" t="inlineStr">
+      <c r="D62" t="n">
+        <v>62</v>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -13543,7 +14043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13556,14 +14056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:47:44</t>
+          <t>Última actualización: 18:15:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 59</t>
+          <t>Total filas: 62</t>
         </is>
       </c>
     </row>
@@ -14947,12 +15447,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>18:29</t>
+          <t>18:26</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -14961,7 +15461,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -14972,37 +15472,37 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:29</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>89</v>
+        <v>42</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>18:31</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -15011,7 +15511,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>109</v>
+        <v>89</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -15022,12 +15522,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>18:31</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -15036,7 +15536,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>52</v>
+        <v>109</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -15052,18 +15552,93 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
+          <t>18:39</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>52</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>30</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D64" t="n">
+      <c r="D66" t="n">
         <v>63</v>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>18:58</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>43</v>
+      </c>
+      <c r="E67" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1776
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E488"/>
+  <dimension ref="A1:E507"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:15:10</t>
+          <t>Última actualización: 18:46:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 483</t>
+          <t>Total filas: 502</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>113</v>
+        <v>40</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4248,7 +4248,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4258,11 +4258,11 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>95</v>
+        <v>40</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4633,7 +4633,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4858,7 +4858,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5208,11 +5208,11 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D223" t="n">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6908,7 +6908,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6933,11 +6933,11 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_RUTA 36_ESC 70</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,7 +6948,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -6958,11 +6958,11 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>92</v>
+        <v>6</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6998,7 +6998,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -7008,11 +7008,11 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>6</v>
+        <v>92</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7283,7 +7283,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D278" t="n">
@@ -7308,7 +7308,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D279" t="n">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D289" t="n">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>5</v>
+        <v>62</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D330" t="n">
@@ -8723,7 +8723,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -8733,11 +8733,11 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,7 +8748,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
@@ -8758,11 +8758,11 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -9048,7 +9048,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -9058,11 +9058,11 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,7 +9073,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -9083,11 +9083,11 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D352" t="n">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D353" t="n">
@@ -9308,7 +9308,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D359" t="n">
@@ -9323,7 +9323,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
@@ -9333,11 +9333,11 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -9358,7 +9358,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -9373,7 +9373,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -9383,11 +9383,11 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -9408,7 +9408,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D363" t="n">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D365" t="n">
@@ -9533,7 +9533,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D368" t="n">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D369" t="n">
@@ -9683,7 +9683,7 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D374" t="n">
@@ -9708,7 +9708,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D375" t="n">
@@ -10023,7 +10023,7 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
@@ -10033,11 +10033,11 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>104</v>
+        <v>45</v>
       </c>
       <c r="E388" t="inlineStr">
         <is>
@@ -10048,7 +10048,7 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
@@ -10058,11 +10058,11 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>45</v>
+        <v>104</v>
       </c>
       <c r="E389" t="inlineStr">
         <is>
@@ -10123,7 +10123,7 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
@@ -10133,11 +10133,11 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>11</v>
+        <v>109</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -10148,7 +10148,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
@@ -10158,11 +10158,11 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>109</v>
+        <v>11</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -10533,7 +10533,7 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D408" t="n">
@@ -10558,7 +10558,7 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D409" t="n">
@@ -10583,7 +10583,7 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D410" t="n">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D411" t="n">
@@ -10633,7 +10633,7 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D412" t="n">
@@ -10658,7 +10658,7 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D413" t="n">
@@ -10683,7 +10683,7 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D414" t="n">
@@ -11048,7 +11048,7 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
@@ -11058,11 +11058,11 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D429" t="n">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="E429" t="inlineStr">
         <is>
@@ -11073,7 +11073,7 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
@@ -11083,11 +11083,11 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D430" t="n">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="E430" t="inlineStr">
         <is>
@@ -11283,7 +11283,7 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D438" t="n">
@@ -11308,7 +11308,7 @@
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D439" t="n">
@@ -11548,7 +11548,7 @@
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
@@ -11558,11 +11558,11 @@
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D449" t="n">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="E449" t="inlineStr">
         <is>
@@ -11573,7 +11573,7 @@
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
@@ -11583,11 +11583,11 @@
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D450" t="n">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="E450" t="inlineStr">
         <is>
@@ -11608,7 +11608,7 @@
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D451" t="n">
@@ -11633,7 +11633,7 @@
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D452" t="n">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D453" t="n">
@@ -11683,7 +11683,7 @@
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D454" t="n">
@@ -11708,7 +11708,7 @@
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D455" t="n">
@@ -11998,21 +11998,21 @@
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>18:49</t>
+          <t>18:46</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D467" t="n">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="E467" t="inlineStr">
         <is>
@@ -12023,12 +12023,12 @@
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>18:49</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
@@ -12037,7 +12037,7 @@
         </is>
       </c>
       <c r="D468" t="n">
-        <v>63</v>
+        <v>108</v>
       </c>
       <c r="E468" t="inlineStr">
         <is>
@@ -12048,21 +12048,21 @@
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:50</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D469" t="n">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="E469" t="inlineStr">
         <is>
@@ -12078,16 +12078,16 @@
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D470" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E470" t="inlineStr">
         <is>
@@ -12098,21 +12098,21 @@
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>19:07</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D471" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="E471" t="inlineStr">
         <is>
@@ -12123,21 +12123,21 @@
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C472" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D472" t="n">
-        <v>53</v>
+        <v>9</v>
       </c>
       <c r="E472" t="inlineStr">
         <is>
@@ -12148,21 +12148,21 @@
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>18:56</t>
         </is>
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D473" t="n">
-        <v>84</v>
+        <v>10</v>
       </c>
       <c r="E473" t="inlineStr">
         <is>
@@ -12173,21 +12173,21 @@
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:01</t>
         </is>
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D474" t="n">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="E474" t="inlineStr">
         <is>
@@ -12198,21 +12198,21 @@
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D475" t="n">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="E475" t="inlineStr">
         <is>
@@ -12223,21 +12223,21 @@
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D476" t="n">
-        <v>63</v>
+        <v>22</v>
       </c>
       <c r="E476" t="inlineStr">
         <is>
@@ -12248,21 +12248,21 @@
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D477" t="n">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="E477" t="inlineStr">
         <is>
@@ -12273,21 +12273,21 @@
     <row r="478">
       <c r="A478" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D478" t="n">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="E478" t="inlineStr">
         <is>
@@ -12298,21 +12298,21 @@
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D479" t="n">
-        <v>94</v>
+        <v>31</v>
       </c>
       <c r="E479" t="inlineStr">
         <is>
@@ -12323,21 +12323,21 @@
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D480" t="n">
-        <v>96</v>
+        <v>32</v>
       </c>
       <c r="E480" t="inlineStr">
         <is>
@@ -12348,21 +12348,21 @@
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D481" t="n">
-        <v>97</v>
+        <v>33</v>
       </c>
       <c r="E481" t="inlineStr">
         <is>
@@ -12373,21 +12373,21 @@
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>19:28</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D482" t="n">
-        <v>101</v>
+        <v>33</v>
       </c>
       <c r="E482" t="inlineStr">
         <is>
@@ -12403,16 +12403,16 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D483" t="n">
-        <v>81</v>
+        <v>64</v>
       </c>
       <c r="E483" t="inlineStr">
         <is>
@@ -12423,21 +12423,21 @@
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D484" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="E484" t="inlineStr">
         <is>
@@ -12448,21 +12448,21 @@
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>19:48</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D485" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E485" t="inlineStr">
         <is>
@@ -12473,21 +12473,21 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>19:51</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D486" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E486" t="inlineStr">
         <is>
@@ -12498,21 +12498,21 @@
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>19:52</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D487" t="n">
-        <v>97</v>
+        <v>39</v>
       </c>
       <c r="E487" t="inlineStr">
         <is>
@@ -12523,23 +12523,498 @@
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>19:27</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D488" t="n">
+        <v>41</v>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>19:27</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D489" t="n">
+        <v>41</v>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>17:47:44</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>19:28</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D490" t="n">
+        <v>101</v>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
           <t>18:15:10</t>
         </is>
       </c>
-      <c r="B488" t="inlineStr">
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D491" t="n">
+        <v>81</v>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D492" t="n">
+        <v>88</v>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>19:48</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D493" t="n">
+        <v>62</v>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>18:15:10</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>19:51</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D494" t="n">
+        <v>96</v>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>19:52</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D495" t="n">
+        <v>66</v>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>19:54</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D496" t="n">
+        <v>68</v>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
         <is>
           <t>19:58</t>
         </is>
       </c>
-      <c r="C488" t="inlineStr">
+      <c r="C497" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D488" t="n">
-        <v>103</v>
-      </c>
-      <c r="E488" t="inlineStr">
+      <c r="D497" t="n">
+        <v>72</v>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>20:06</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D498" t="n">
+        <v>80</v>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>20:06</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D499" t="n">
+        <v>80</v>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D500" t="n">
+        <v>89</v>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>20:17</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D501" t="n">
+        <v>91</v>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>20:18</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D502" t="n">
+        <v>92</v>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>20:20</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D503" t="n">
+        <v>94</v>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>20:21</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D504" t="n">
+        <v>95</v>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D505" t="n">
+        <v>97</v>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>20:27</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D506" t="n">
+        <v>101</v>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>20:33</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D507" t="n">
+        <v>107</v>
+      </c>
+      <c r="E507" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -12556,7 +13031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12569,14 +13044,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:15:10</t>
+          <t>Última actualización: 18:46:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 57</t>
+          <t>Total filas: 59</t>
         </is>
       </c>
     </row>
@@ -13935,7 +14410,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -13945,11 +14420,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -13960,7 +14435,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -13970,11 +14445,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -14010,7 +14485,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -14024,9 +14499,59 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>20:27</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>101</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>20:33</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>107</v>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -14043,7 +14568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14056,14 +14581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:15:10</t>
+          <t>Última actualización: 18:46:01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 62</t>
+          <t>Total filas: 66</t>
         </is>
       </c>
     </row>
@@ -15639,6 +16164,106 @@
         <v>43</v>
       </c>
       <c r="E67" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>19:01</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>15</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>89</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>20:21</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>95</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>20:36</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>110</v>
+      </c>
+      <c r="E71" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1777
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E507"/>
+  <dimension ref="A1:E529"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:46:01</t>
+          <t>Última actualización: 18:59:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 502</t>
+          <t>Total filas: 524</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -658,11 +658,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -683,11 +683,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1773,7 +1773,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1783,11 +1783,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>18</v>
+        <v>86</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3508,7 +3508,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4248,7 +4248,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4258,11 +4258,11 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>95</v>
+        <v>40</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4633,7 +4633,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4858,7 +4858,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5208,11 +5208,11 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5458,11 +5458,11 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5483,11 +5483,11 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_RUTA 36_ESC 70</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6933,11 +6933,11 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6983,7 +6983,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D266" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D267" t="n">
@@ -7023,7 +7023,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -7033,11 +7033,11 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,7 +7048,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -7058,11 +7058,11 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7158,11 +7158,11 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7198,7 +7198,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -7208,11 +7208,11 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7283,7 +7283,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D278" t="n">
@@ -7308,7 +7308,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D279" t="n">
@@ -7483,7 +7483,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D286" t="n">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D287" t="n">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D305" t="n">
@@ -7983,7 +7983,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D306" t="n">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8323,7 +8323,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -8333,11 +8333,11 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -8358,11 +8358,11 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8433,7 +8433,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D324" t="n">
@@ -8458,7 +8458,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D325" t="n">
@@ -8508,7 +8508,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D327" t="n">
@@ -8533,7 +8533,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D328" t="n">
@@ -8683,7 +8683,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D334" t="n">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D352" t="n">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D353" t="n">
@@ -9333,7 +9333,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D360" t="n">
@@ -9358,7 +9358,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -9408,7 +9408,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D363" t="n">
@@ -9433,7 +9433,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D364" t="n">
@@ -9533,7 +9533,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D368" t="n">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D369" t="n">
@@ -9683,7 +9683,7 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D374" t="n">
@@ -9708,7 +9708,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D375" t="n">
@@ -9883,7 +9883,7 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D382" t="n">
@@ -9908,7 +9908,7 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D383" t="n">
@@ -10023,7 +10023,7 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
@@ -10033,11 +10033,11 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>45</v>
+        <v>104</v>
       </c>
       <c r="E388" t="inlineStr">
         <is>
@@ -10048,7 +10048,7 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
@@ -10058,11 +10058,11 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>104</v>
+        <v>45</v>
       </c>
       <c r="E389" t="inlineStr">
         <is>
@@ -10533,7 +10533,7 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D408" t="n">
@@ -10558,7 +10558,7 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D409" t="n">
@@ -10583,7 +10583,7 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D410" t="n">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D411" t="n">
@@ -10633,7 +10633,7 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D412" t="n">
@@ -10658,7 +10658,7 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D413" t="n">
@@ -10683,7 +10683,7 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D414" t="n">
@@ -11008,7 +11008,7 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D427" t="n">
@@ -11033,7 +11033,7 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D428" t="n">
@@ -11098,7 +11098,7 @@
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
@@ -11108,11 +11108,11 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D431" t="n">
-        <v>112</v>
+        <v>54</v>
       </c>
       <c r="E431" t="inlineStr">
         <is>
@@ -11123,7 +11123,7 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
@@ -11133,11 +11133,11 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D432" t="n">
-        <v>54</v>
+        <v>112</v>
       </c>
       <c r="E432" t="inlineStr">
         <is>
@@ -11198,7 +11198,7 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
@@ -11208,11 +11208,11 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D435" t="n">
-        <v>12</v>
+        <v>58</v>
       </c>
       <c r="E435" t="inlineStr">
         <is>
@@ -11223,7 +11223,7 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
@@ -11233,11 +11233,11 @@
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D436" t="n">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="E436" t="inlineStr">
         <is>
@@ -11573,7 +11573,7 @@
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
@@ -11583,11 +11583,11 @@
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D450" t="n">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="E450" t="inlineStr">
         <is>
@@ -11598,7 +11598,7 @@
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
@@ -11608,11 +11608,11 @@
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D451" t="n">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="E451" t="inlineStr">
         <is>
@@ -12173,12 +12173,12 @@
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>19:01</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C474" t="inlineStr">
@@ -12187,7 +12187,7 @@
         </is>
       </c>
       <c r="D474" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E474" t="inlineStr">
         <is>
@@ -12198,21 +12198,21 @@
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>19:07</t>
+          <t>19:01</t>
         </is>
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D475" t="n">
-        <v>80</v>
+        <v>15</v>
       </c>
       <c r="E475" t="inlineStr">
         <is>
@@ -12223,21 +12223,21 @@
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:03</t>
         </is>
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D476" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="E476" t="inlineStr">
         <is>
@@ -12248,21 +12248,21 @@
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D477" t="n">
-        <v>84</v>
+        <v>8</v>
       </c>
       <c r="E477" t="inlineStr">
         <is>
@@ -12278,16 +12278,16 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C478" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D478" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E478" t="inlineStr">
         <is>
@@ -12298,21 +12298,21 @@
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D479" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="E479" t="inlineStr">
         <is>
@@ -12328,16 +12328,16 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D480" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E480" t="inlineStr">
         <is>
@@ -12348,21 +12348,21 @@
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>19:13</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D481" t="n">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="E481" t="inlineStr">
         <is>
@@ -12373,21 +12373,21 @@
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D482" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="E482" t="inlineStr">
         <is>
@@ -12398,21 +12398,21 @@
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D483" t="n">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="E483" t="inlineStr">
         <is>
@@ -12423,21 +12423,21 @@
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D484" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="E484" t="inlineStr">
         <is>
@@ -12448,21 +12448,21 @@
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:18</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D485" t="n">
-        <v>96</v>
+        <v>32</v>
       </c>
       <c r="E485" t="inlineStr">
         <is>
@@ -12473,21 +12473,21 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D486" t="n">
-        <v>97</v>
+        <v>33</v>
       </c>
       <c r="E486" t="inlineStr">
         <is>
@@ -12498,21 +12498,21 @@
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D487" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="E487" t="inlineStr">
         <is>
@@ -12523,12 +12523,12 @@
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>19:27</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
@@ -12537,7 +12537,7 @@
         </is>
       </c>
       <c r="D488" t="n">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="E488" t="inlineStr">
         <is>
@@ -12548,21 +12548,21 @@
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>19:27</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D489" t="n">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="E489" t="inlineStr">
         <is>
@@ -12578,16 +12578,16 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>19:28</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D490" t="n">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="E490" t="inlineStr">
         <is>
@@ -12598,21 +12598,21 @@
     <row r="491">
       <c r="A491" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D491" t="n">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="E491" t="inlineStr">
         <is>
@@ -12623,21 +12623,21 @@
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D492" t="n">
-        <v>88</v>
+        <v>25</v>
       </c>
       <c r="E492" t="inlineStr">
         <is>
@@ -12648,21 +12648,21 @@
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>19:48</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D493" t="n">
-        <v>62</v>
+        <v>97</v>
       </c>
       <c r="E493" t="inlineStr">
         <is>
@@ -12673,21 +12673,21 @@
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>19:51</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D494" t="n">
-        <v>96</v>
+        <v>39</v>
       </c>
       <c r="E494" t="inlineStr">
         <is>
@@ -12698,21 +12698,21 @@
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>19:52</t>
+          <t>19:26</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D495" t="n">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="E495" t="inlineStr">
         <is>
@@ -12728,16 +12728,16 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:27</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D496" t="n">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="E496" t="inlineStr">
         <is>
@@ -12753,16 +12753,16 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>19:58</t>
+          <t>19:27</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D497" t="n">
-        <v>72</v>
+        <v>41</v>
       </c>
       <c r="E497" t="inlineStr">
         <is>
@@ -12773,21 +12773,21 @@
     <row r="498">
       <c r="A498" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>19:28</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D498" t="n">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="E498" t="inlineStr">
         <is>
@@ -12798,12 +12798,12 @@
     <row r="499">
       <c r="A499" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>19:33</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
@@ -12812,7 +12812,7 @@
         </is>
       </c>
       <c r="D499" t="n">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="E499" t="inlineStr">
         <is>
@@ -12823,12 +12823,12 @@
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:36</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
@@ -12837,7 +12837,7 @@
         </is>
       </c>
       <c r="D500" t="n">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="E500" t="inlineStr">
         <is>
@@ -12848,21 +12848,21 @@
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>20:17</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D501" t="n">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E501" t="inlineStr">
         <is>
@@ -12873,21 +12873,21 @@
     <row r="502">
       <c r="A502" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>20:18</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D502" t="n">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="E502" t="inlineStr">
         <is>
@@ -12898,21 +12898,21 @@
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>20:20</t>
+          <t>19:46</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D503" t="n">
-        <v>94</v>
+        <v>47</v>
       </c>
       <c r="E503" t="inlineStr">
         <is>
@@ -12923,21 +12923,21 @@
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>20:21</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D504" t="n">
-        <v>95</v>
+        <v>48</v>
       </c>
       <c r="E504" t="inlineStr">
         <is>
@@ -12953,16 +12953,16 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>19:48</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D505" t="n">
-        <v>97</v>
+        <v>62</v>
       </c>
       <c r="E505" t="inlineStr">
         <is>
@@ -12973,21 +12973,21 @@
     <row r="506">
       <c r="A506" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>19:51</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D506" t="n">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E506" t="inlineStr">
         <is>
@@ -12998,23 +12998,573 @@
     <row r="507">
       <c r="A507" t="inlineStr">
         <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>19:51</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D507" t="n">
+        <v>52</v>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
           <t>18:46:01</t>
         </is>
       </c>
-      <c r="B507" t="inlineStr">
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>19:52</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D508" t="n">
+        <v>66</v>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>19:54</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D509" t="n">
+        <v>68</v>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>19:57</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D510" t="n">
+        <v>58</v>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>19:58</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D511" t="n">
+        <v>72</v>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D512" t="n">
+        <v>66</v>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>20:06</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D513" t="n">
+        <v>80</v>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>20:06</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D514" t="n">
+        <v>80</v>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>20:11</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D515" t="n">
+        <v>72</v>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D516" t="n">
+        <v>89</v>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>20:17</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D517" t="n">
+        <v>78</v>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>20:17</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D518" t="n">
+        <v>91</v>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>20:18</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D519" t="n">
+        <v>92</v>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>20:20</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D520" t="n">
+        <v>81</v>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>20:21</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D521" t="n">
+        <v>95</v>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D522" t="n">
+        <v>84</v>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>20:27</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D523" t="n">
+        <v>88</v>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>20:29</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D524" t="n">
+        <v>90</v>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>20:32</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D525" t="n">
+        <v>93</v>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
         <is>
           <t>20:33</t>
         </is>
       </c>
-      <c r="C507" t="inlineStr">
+      <c r="C526" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D507" t="n">
+      <c r="D526" t="n">
         <v>107</v>
       </c>
-      <c r="E507" t="inlineStr">
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>20:46</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D527" t="n">
+        <v>107</v>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>20:54</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D528" t="n">
+        <v>115</v>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D529" t="n">
+        <v>118</v>
+      </c>
+      <c r="E529" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -13031,7 +13581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13044,14 +13594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:46:01</t>
+          <t>Última actualización: 18:59:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 59</t>
+          <t>Total filas: 61</t>
         </is>
       </c>
     </row>
@@ -14410,7 +14960,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -14420,11 +14970,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -14435,7 +14985,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -14445,11 +14995,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -14485,7 +15035,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -14499,7 +15049,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -14510,7 +15060,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -14524,7 +15074,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -14535,23 +15085,73 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>20:32</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>93</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>18:46:01</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>20:33</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D64" t="n">
+      <c r="D65" t="n">
         <v>107</v>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>20:54</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>115</v>
+      </c>
+      <c r="E66" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -14568,7 +15168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14581,14 +15181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:46:01</t>
+          <t>Última actualización: 18:59:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 66</t>
+          <t>Total filas: 71</t>
         </is>
       </c>
     </row>
@@ -16197,50 +16797,50 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:03</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>89</v>
+        <v>4</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>20:21</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
@@ -16252,20 +16852,145 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>89</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>20:20</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>81</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>20:21</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>95</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>96</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
           <t>20:36</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D71" t="n">
+      <c r="D75" t="n">
         <v>110</v>
       </c>
-      <c r="E71" t="inlineStr">
+      <c r="E75" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>20:54</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>115</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1778
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E529"/>
+  <dimension ref="A1:E545"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:59:44</t>
+          <t>Última actualización: 19:29:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 524</t>
+          <t>Total filas: 540</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>22</v>
+        <v>113</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>95</v>
+        <v>40</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,7 +4748,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -4758,11 +4758,11 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>5</v>
+        <v>65</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4858,7 +4858,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5208,11 +5208,11 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5458,11 +5458,11 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5483,11 +5483,11 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6933,11 +6933,11 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_RUTA 36_ESC 70</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6983,7 +6983,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D266" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D267" t="n">
@@ -7023,7 +7023,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -7033,11 +7033,11 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,7 +7048,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -7058,11 +7058,11 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D289" t="n">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -8258,7 +8258,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D317" t="n">
@@ -8283,7 +8283,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D318" t="n">
@@ -8483,7 +8483,7 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D326" t="n">
@@ -8508,7 +8508,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D327" t="n">
@@ -8723,7 +8723,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -8733,11 +8733,11 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,7 +8748,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
@@ -8758,11 +8758,11 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D352" t="n">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D353" t="n">
@@ -9408,7 +9408,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D363" t="n">
@@ -9433,7 +9433,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D364" t="n">
@@ -9533,7 +9533,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D368" t="n">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D369" t="n">
@@ -9883,7 +9883,7 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D382" t="n">
@@ -9908,7 +9908,7 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D383" t="n">
@@ -9923,7 +9923,7 @@
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
@@ -9933,11 +9933,11 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="E384" t="inlineStr">
         <is>
@@ -9948,7 +9948,7 @@
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
@@ -9958,11 +9958,11 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="E385" t="inlineStr">
         <is>
@@ -10023,7 +10023,7 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
@@ -10033,11 +10033,11 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>104</v>
+        <v>45</v>
       </c>
       <c r="E388" t="inlineStr">
         <is>
@@ -10048,7 +10048,7 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
@@ -10058,11 +10058,11 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>45</v>
+        <v>104</v>
       </c>
       <c r="E389" t="inlineStr">
         <is>
@@ -10123,7 +10123,7 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
@@ -10133,11 +10133,11 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>109</v>
+        <v>11</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -10148,7 +10148,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
@@ -10158,11 +10158,11 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>11</v>
+        <v>109</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -10273,7 +10273,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
@@ -10283,11 +10283,11 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E398" t="inlineStr">
         <is>
@@ -10298,7 +10298,7 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
@@ -10308,11 +10308,11 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D399" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E399" t="inlineStr">
         <is>
@@ -10333,7 +10333,7 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D400" t="n">
@@ -10533,7 +10533,7 @@
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D408" t="n">
@@ -10558,7 +10558,7 @@
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D409" t="n">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D411" t="n">
@@ -10633,7 +10633,7 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D412" t="n">
@@ -10658,7 +10658,7 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D413" t="n">
@@ -10683,7 +10683,7 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D414" t="n">
@@ -10798,7 +10798,7 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
@@ -10808,11 +10808,11 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D419" t="n">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E419" t="inlineStr">
         <is>
@@ -10823,7 +10823,7 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
@@ -10833,11 +10833,11 @@
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D420" t="n">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="E420" t="inlineStr">
         <is>
@@ -10958,7 +10958,7 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D425" t="n">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D426" t="n">
@@ -11008,7 +11008,7 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D427" t="n">
@@ -11033,7 +11033,7 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D428" t="n">
@@ -11098,7 +11098,7 @@
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
@@ -11108,11 +11108,11 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D431" t="n">
-        <v>54</v>
+        <v>112</v>
       </c>
       <c r="E431" t="inlineStr">
         <is>
@@ -11123,7 +11123,7 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
@@ -11133,11 +11133,11 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D432" t="n">
-        <v>112</v>
+        <v>54</v>
       </c>
       <c r="E432" t="inlineStr">
         <is>
@@ -11198,7 +11198,7 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
@@ -11208,11 +11208,11 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D435" t="n">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="E435" t="inlineStr">
         <is>
@@ -11223,7 +11223,7 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
@@ -11233,11 +11233,11 @@
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D436" t="n">
-        <v>12</v>
+        <v>58</v>
       </c>
       <c r="E436" t="inlineStr">
         <is>
@@ -11283,7 +11283,7 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D438" t="n">
@@ -11308,7 +11308,7 @@
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D439" t="n">
@@ -11548,7 +11548,7 @@
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
@@ -11558,11 +11558,11 @@
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D449" t="n">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="E449" t="inlineStr">
         <is>
@@ -11583,7 +11583,7 @@
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D450" t="n">
@@ -11598,7 +11598,7 @@
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
@@ -11608,11 +11608,11 @@
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D451" t="n">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="E451" t="inlineStr">
         <is>
@@ -11633,7 +11633,7 @@
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D452" t="n">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D453" t="n">
@@ -11683,7 +11683,7 @@
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D454" t="n">
@@ -11708,7 +11708,7 @@
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D455" t="n">
@@ -11898,7 +11898,7 @@
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B463" t="inlineStr">
@@ -11908,11 +11908,11 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D463" t="n">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="E463" t="inlineStr">
         <is>
@@ -11923,7 +11923,7 @@
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
@@ -11933,11 +11933,11 @@
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D464" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="E464" t="inlineStr">
         <is>
@@ -12383,7 +12383,7 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D482" t="n">
@@ -12408,7 +12408,7 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D483" t="n">
@@ -12423,7 +12423,7 @@
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
@@ -12433,11 +12433,11 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D484" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="E484" t="inlineStr">
         <is>
@@ -12448,7 +12448,7 @@
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B485" t="inlineStr">
@@ -12458,11 +12458,11 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D485" t="n">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="E485" t="inlineStr">
         <is>
@@ -12498,7 +12498,7 @@
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
@@ -12508,11 +12508,11 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D487" t="n">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="E487" t="inlineStr">
         <is>
@@ -12523,7 +12523,7 @@
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
@@ -12533,11 +12533,11 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D488" t="n">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="E488" t="inlineStr">
         <is>
@@ -12798,21 +12798,21 @@
     <row r="499">
       <c r="A499" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>19:33</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D499" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E499" t="inlineStr">
         <is>
@@ -12823,21 +12823,21 @@
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D500" t="n">
-        <v>81</v>
+        <v>1</v>
       </c>
       <c r="E500" t="inlineStr">
         <is>
@@ -12848,21 +12848,21 @@
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:33</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D501" t="n">
-        <v>88</v>
+        <v>34</v>
       </c>
       <c r="E501" t="inlineStr">
         <is>
@@ -12873,21 +12873,21 @@
     <row r="502">
       <c r="A502" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:36</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D502" t="n">
-        <v>44</v>
+        <v>81</v>
       </c>
       <c r="E502" t="inlineStr">
         <is>
@@ -12898,21 +12898,21 @@
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D503" t="n">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="E503" t="inlineStr">
         <is>
@@ -12923,21 +12923,21 @@
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D504" t="n">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="E504" t="inlineStr">
         <is>
@@ -12948,21 +12948,21 @@
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>19:48</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D505" t="n">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="E505" t="inlineStr">
         <is>
@@ -12973,21 +12973,21 @@
     <row r="506">
       <c r="A506" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>19:51</t>
+          <t>19:46</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D506" t="n">
-        <v>96</v>
+        <v>47</v>
       </c>
       <c r="E506" t="inlineStr">
         <is>
@@ -12998,21 +12998,21 @@
     <row r="507">
       <c r="A507" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>19:51</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D507" t="n">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="E507" t="inlineStr">
         <is>
@@ -13028,16 +13028,16 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>19:52</t>
+          <t>19:48</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D508" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E508" t="inlineStr">
         <is>
@@ -13048,21 +13048,21 @@
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:51</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D509" t="n">
-        <v>68</v>
+        <v>22</v>
       </c>
       <c r="E509" t="inlineStr">
         <is>
@@ -13073,12 +13073,12 @@
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>19:57</t>
+          <t>19:51</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
@@ -13087,7 +13087,7 @@
         </is>
       </c>
       <c r="D510" t="n">
-        <v>58</v>
+        <v>96</v>
       </c>
       <c r="E510" t="inlineStr">
         <is>
@@ -13103,16 +13103,16 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>19:58</t>
+          <t>19:52</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D511" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="E511" t="inlineStr">
         <is>
@@ -13123,21 +13123,21 @@
     <row r="512">
       <c r="A512" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>19:54</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D512" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E512" t="inlineStr">
         <is>
@@ -13148,21 +13148,21 @@
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>19:57</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D513" t="n">
-        <v>80</v>
+        <v>28</v>
       </c>
       <c r="E513" t="inlineStr">
         <is>
@@ -13173,21 +13173,21 @@
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>19:58</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D514" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E514" t="inlineStr">
         <is>
@@ -13198,17 +13198,17 @@
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>20:11</t>
+          <t>19:58</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D515" t="n">
@@ -13223,21 +13223,21 @@
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D516" t="n">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="E516" t="inlineStr">
         <is>
@@ -13248,21 +13248,21 @@
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>20:17</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D517" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E517" t="inlineStr">
         <is>
@@ -13278,16 +13278,16 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>20:17</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D518" t="n">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="E518" t="inlineStr">
         <is>
@@ -13298,21 +13298,21 @@
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>20:18</t>
+          <t>20:11</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D519" t="n">
-        <v>92</v>
+        <v>42</v>
       </c>
       <c r="E519" t="inlineStr">
         <is>
@@ -13323,21 +13323,21 @@
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>20:20</t>
+          <t>20:13</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D520" t="n">
-        <v>81</v>
+        <v>44</v>
       </c>
       <c r="E520" t="inlineStr">
         <is>
@@ -13353,16 +13353,16 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>20:21</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D521" t="n">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E521" t="inlineStr">
         <is>
@@ -13373,21 +13373,21 @@
     <row r="522">
       <c r="A522" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:17</t>
         </is>
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D522" t="n">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="E522" t="inlineStr">
         <is>
@@ -13398,21 +13398,21 @@
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:17</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D523" t="n">
-        <v>88</v>
+        <v>48</v>
       </c>
       <c r="E523" t="inlineStr">
         <is>
@@ -13423,21 +13423,21 @@
     <row r="524">
       <c r="A524" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>20:29</t>
+          <t>20:18</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D524" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E524" t="inlineStr">
         <is>
@@ -13448,21 +13448,21 @@
     <row r="525">
       <c r="A525" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:20</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D525" t="n">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="E525" t="inlineStr">
         <is>
@@ -13478,16 +13478,16 @@
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>20:33</t>
+          <t>20:21</t>
         </is>
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D526" t="n">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="E526" t="inlineStr">
         <is>
@@ -13498,21 +13498,21 @@
     <row r="527">
       <c r="A527" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>20:46</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D527" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E527" t="inlineStr">
         <is>
@@ -13523,21 +13523,21 @@
     <row r="528">
       <c r="A528" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>20:54</t>
+          <t>20:26</t>
         </is>
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D528" t="n">
-        <v>115</v>
+        <v>57</v>
       </c>
       <c r="E528" t="inlineStr">
         <is>
@@ -13553,18 +13553,418 @@
       </c>
       <c r="B529" t="inlineStr">
         <is>
+          <t>20:27</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D529" t="n">
+        <v>88</v>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>20:29</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D530" t="n">
+        <v>90</v>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>20:32</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D531" t="n">
+        <v>63</v>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>20:33</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D532" t="n">
+        <v>107</v>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>20:37</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D533" t="n">
+        <v>68</v>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D534" t="n">
+        <v>71</v>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D535" t="n">
+        <v>76</v>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>20:46</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D536" t="n">
+        <v>107</v>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>20:53</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D537" t="n">
+        <v>84</v>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>20:54</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D538" t="n">
+        <v>115</v>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D539" t="n">
+        <v>87</v>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
           <t>20:57</t>
         </is>
       </c>
-      <c r="C529" t="inlineStr">
+      <c r="C540" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D529" t="n">
+      <c r="D540" t="n">
         <v>118</v>
       </c>
-      <c r="E529" t="inlineStr">
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>20:58</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D541" t="n">
+        <v>89</v>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>20:58</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D542" t="n">
+        <v>89</v>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>21:01</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D543" t="n">
+        <v>92</v>
+      </c>
+      <c r="E543" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D544" t="n">
+        <v>97</v>
+      </c>
+      <c r="E544" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>21:20</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D545" t="n">
+        <v>111</v>
+      </c>
+      <c r="E545" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -13581,7 +13981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13594,14 +13994,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:59:44</t>
+          <t>Última actualización: 19:29:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 61</t>
+          <t>Total filas: 63</t>
         </is>
       </c>
     </row>
@@ -15060,12 +15460,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:26</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -15074,7 +15474,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>88</v>
+        <v>57</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -15090,16 +15490,16 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:27</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -15110,12 +15510,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>20:33</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -15124,7 +15524,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>107</v>
+        <v>63</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -15135,23 +15535,73 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>18:46:01</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>20:33</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>107</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>71</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
           <t>18:59:44</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>20:54</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D66" t="n">
+      <c r="D68" t="n">
         <v>115</v>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E68" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -15181,7 +15631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:59:44</t>
+          <t>Última actualización: 19:29:54</t>
         </is>
       </c>
     </row>
@@ -16822,7 +17272,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -16836,7 +17286,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -16872,7 +17322,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -16886,7 +17336,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>81</v>
+        <v>51</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -16922,7 +17372,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -16936,7 +17386,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>96</v>
+        <v>66</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -16972,7 +17422,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -16986,7 +17436,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1779
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E545"/>
+  <dimension ref="A1:E562"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:29:54</t>
+          <t>Última actualización: 19:56:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 540</t>
+          <t>Total filas: 557</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -658,11 +658,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -683,11 +683,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>22</v>
+        <v>113</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>40</v>
+        <v>95</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,7 +4523,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4533,11 +4533,11 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>95</v>
+        <v>40</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4858,7 +4858,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5208,11 +5208,11 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5458,11 +5458,11 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5483,11 +5483,11 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D223" t="n">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_RUTA 36_ESC 70</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6933,11 +6933,11 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -7283,7 +7283,7 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D278" t="n">
@@ -7308,7 +7308,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D279" t="n">
@@ -7483,7 +7483,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D286" t="n">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D287" t="n">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D289" t="n">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>5</v>
+        <v>62</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -8323,7 +8323,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -8333,11 +8333,11 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -8358,11 +8358,11 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8433,7 +8433,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D324" t="n">
@@ -8458,7 +8458,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D325" t="n">
@@ -8483,7 +8483,7 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D326" t="n">
@@ -8508,7 +8508,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D327" t="n">
@@ -8533,7 +8533,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D328" t="n">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D330" t="n">
@@ -8683,7 +8683,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D334" t="n">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -8723,7 +8723,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -8733,11 +8733,11 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,7 +8748,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
@@ -8758,11 +8758,11 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -9048,7 +9048,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -9058,11 +9058,11 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,7 +9073,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -9083,11 +9083,11 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D352" t="n">
@@ -9158,7 +9158,7 @@
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D353" t="n">
@@ -9308,7 +9308,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D359" t="n">
@@ -9358,7 +9358,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -9433,7 +9433,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D364" t="n">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D365" t="n">
@@ -9533,7 +9533,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D368" t="n">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D369" t="n">
@@ -9683,7 +9683,7 @@
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D374" t="n">
@@ -9708,7 +9708,7 @@
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D375" t="n">
@@ -10083,7 +10083,7 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D390" t="n">
@@ -10108,7 +10108,7 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D391" t="n">
@@ -10123,7 +10123,7 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
@@ -10133,11 +10133,11 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>11</v>
+        <v>109</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -10148,7 +10148,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
@@ -10158,11 +10158,11 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>109</v>
+        <v>11</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -10273,7 +10273,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
@@ -10283,11 +10283,11 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E398" t="inlineStr">
         <is>
@@ -10308,7 +10308,7 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D399" t="n">
@@ -10323,7 +10323,7 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
@@ -10333,11 +10333,11 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D400" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E400" t="inlineStr">
         <is>
@@ -10398,7 +10398,7 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
@@ -10408,11 +10408,11 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D403" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E403" t="inlineStr">
         <is>
@@ -10423,7 +10423,7 @@
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
@@ -10433,11 +10433,11 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D404" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="E404" t="inlineStr">
         <is>
@@ -10583,7 +10583,7 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D410" t="n">
@@ -10608,7 +10608,7 @@
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D411" t="n">
@@ -10658,7 +10658,7 @@
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D413" t="n">
@@ -10683,7 +10683,7 @@
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D414" t="n">
@@ -11008,7 +11008,7 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D427" t="n">
@@ -11033,7 +11033,7 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D428" t="n">
@@ -11048,7 +11048,7 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
@@ -11058,11 +11058,11 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D429" t="n">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="E429" t="inlineStr">
         <is>
@@ -11073,7 +11073,7 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
@@ -11083,11 +11083,11 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D430" t="n">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="E430" t="inlineStr">
         <is>
@@ -11198,7 +11198,7 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
@@ -11208,11 +11208,11 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D435" t="n">
-        <v>12</v>
+        <v>58</v>
       </c>
       <c r="E435" t="inlineStr">
         <is>
@@ -11223,7 +11223,7 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
@@ -11233,11 +11233,11 @@
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D436" t="n">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="E436" t="inlineStr">
         <is>
@@ -11423,7 +11423,7 @@
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
@@ -11433,11 +11433,11 @@
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D444" t="n">
-        <v>66</v>
+        <v>20</v>
       </c>
       <c r="E444" t="inlineStr">
         <is>
@@ -11448,7 +11448,7 @@
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
@@ -11458,11 +11458,11 @@
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D445" t="n">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="E445" t="inlineStr">
         <is>
@@ -11633,7 +11633,7 @@
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D452" t="n">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D453" t="n">
@@ -11898,7 +11898,7 @@
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B463" t="inlineStr">
@@ -11908,11 +11908,11 @@
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D463" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="E463" t="inlineStr">
         <is>
@@ -11923,7 +11923,7 @@
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
@@ -11933,11 +11933,11 @@
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D464" t="n">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="E464" t="inlineStr">
         <is>
@@ -12383,7 +12383,7 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D482" t="n">
@@ -12408,7 +12408,7 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D483" t="n">
@@ -12423,7 +12423,7 @@
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
@@ -12433,11 +12433,11 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D484" t="n">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="E484" t="inlineStr">
         <is>
@@ -12448,7 +12448,7 @@
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B485" t="inlineStr">
@@ -12458,11 +12458,11 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D485" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="E485" t="inlineStr">
         <is>
@@ -12473,7 +12473,7 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
@@ -12483,11 +12483,11 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D486" t="n">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="E486" t="inlineStr">
         <is>
@@ -12498,7 +12498,7 @@
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
@@ -12508,11 +12508,11 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D487" t="n">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="E487" t="inlineStr">
         <is>
@@ -12523,7 +12523,7 @@
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
@@ -12533,11 +12533,11 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D488" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="E488" t="inlineStr">
         <is>
@@ -12548,7 +12548,7 @@
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B489" t="inlineStr">
@@ -12558,11 +12558,11 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D489" t="n">
-        <v>22</v>
+        <v>94</v>
       </c>
       <c r="E489" t="inlineStr">
         <is>
@@ -12573,7 +12573,7 @@
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B490" t="inlineStr">
@@ -12583,11 +12583,11 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D490" t="n">
-        <v>94</v>
+        <v>22</v>
       </c>
       <c r="E490" t="inlineStr">
         <is>
@@ -13173,21 +13173,21 @@
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>19:58</t>
+          <t>19:57</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D514" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="E514" t="inlineStr">
         <is>
@@ -13198,7 +13198,7 @@
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B515" t="inlineStr">
@@ -13208,11 +13208,11 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D515" t="n">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="E515" t="inlineStr">
         <is>
@@ -13223,21 +13223,21 @@
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>20:05</t>
+          <t>19:58</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D516" t="n">
-        <v>66</v>
+        <v>2</v>
       </c>
       <c r="E516" t="inlineStr">
         <is>
@@ -13248,21 +13248,21 @@
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>19:59</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D517" t="n">
-        <v>80</v>
+        <v>3</v>
       </c>
       <c r="E517" t="inlineStr">
         <is>
@@ -13273,21 +13273,21 @@
     <row r="518">
       <c r="A518" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>20:06</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D518" t="n">
-        <v>80</v>
+        <v>5</v>
       </c>
       <c r="E518" t="inlineStr">
         <is>
@@ -13298,21 +13298,21 @@
     <row r="519">
       <c r="A519" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>20:11</t>
+          <t>20:05</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D519" t="n">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="E519" t="inlineStr">
         <is>
@@ -13323,21 +13323,21 @@
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>20:13</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D520" t="n">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="E520" t="inlineStr">
         <is>
@@ -13353,16 +13353,16 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:06</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D521" t="n">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="E521" t="inlineStr">
         <is>
@@ -13373,21 +13373,21 @@
     <row r="522">
       <c r="A522" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>20:17</t>
+          <t>20:07</t>
         </is>
       </c>
       <c r="C522" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D522" t="n">
-        <v>91</v>
+        <v>11</v>
       </c>
       <c r="E522" t="inlineStr">
         <is>
@@ -13398,21 +13398,21 @@
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>20:17</t>
+          <t>20:09</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D523" t="n">
-        <v>48</v>
+        <v>13</v>
       </c>
       <c r="E523" t="inlineStr">
         <is>
@@ -13423,21 +13423,21 @@
     <row r="524">
       <c r="A524" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>20:18</t>
+          <t>20:11</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D524" t="n">
-        <v>92</v>
+        <v>42</v>
       </c>
       <c r="E524" t="inlineStr">
         <is>
@@ -13448,21 +13448,21 @@
     <row r="525">
       <c r="A525" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>20:20</t>
+          <t>20:12</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D525" t="n">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="E525" t="inlineStr">
         <is>
@@ -13473,21 +13473,21 @@
     <row r="526">
       <c r="A526" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>20:21</t>
+          <t>20:13</t>
         </is>
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D526" t="n">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="E526" t="inlineStr">
         <is>
@@ -13498,21 +13498,21 @@
     <row r="527">
       <c r="A527" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D527" t="n">
-        <v>54</v>
+        <v>89</v>
       </c>
       <c r="E527" t="inlineStr">
         <is>
@@ -13523,21 +13523,21 @@
     <row r="528">
       <c r="A528" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>20:17</t>
         </is>
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D528" t="n">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="E528" t="inlineStr">
         <is>
@@ -13548,21 +13548,21 @@
     <row r="529">
       <c r="A529" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:17</t>
         </is>
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D529" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E529" t="inlineStr">
         <is>
@@ -13573,21 +13573,21 @@
     <row r="530">
       <c r="A530" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>20:29</t>
+          <t>20:18</t>
         </is>
       </c>
       <c r="C530" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D530" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E530" t="inlineStr">
         <is>
@@ -13603,16 +13603,16 @@
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:20</t>
         </is>
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D531" t="n">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="E531" t="inlineStr">
         <is>
@@ -13623,21 +13623,21 @@
     <row r="532">
       <c r="A532" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>20:33</t>
+          <t>20:21</t>
         </is>
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D532" t="n">
-        <v>107</v>
+        <v>25</v>
       </c>
       <c r="E532" t="inlineStr">
         <is>
@@ -13648,21 +13648,21 @@
     <row r="533">
       <c r="A533" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B533" t="inlineStr">
         <is>
-          <t>20:37</t>
+          <t>20:21</t>
         </is>
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D533" t="n">
-        <v>68</v>
+        <v>95</v>
       </c>
       <c r="E533" t="inlineStr">
         <is>
@@ -13673,21 +13673,21 @@
     <row r="534">
       <c r="A534" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B534" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D534" t="n">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="E534" t="inlineStr">
         <is>
@@ -13703,16 +13703,16 @@
       </c>
       <c r="B535" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:26</t>
         </is>
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D535" t="n">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="E535" t="inlineStr">
         <is>
@@ -13723,21 +13723,21 @@
     <row r="536">
       <c r="A536" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B536" t="inlineStr">
         <is>
-          <t>20:46</t>
+          <t>20:27</t>
         </is>
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D536" t="n">
-        <v>107</v>
+        <v>31</v>
       </c>
       <c r="E536" t="inlineStr">
         <is>
@@ -13748,12 +13748,12 @@
     <row r="537">
       <c r="A537" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>20:53</t>
+          <t>20:29</t>
         </is>
       </c>
       <c r="C537" t="inlineStr">
@@ -13762,7 +13762,7 @@
         </is>
       </c>
       <c r="D537" t="n">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="E537" t="inlineStr">
         <is>
@@ -13773,21 +13773,21 @@
     <row r="538">
       <c r="A538" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>20:54</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D538" t="n">
-        <v>115</v>
+        <v>36</v>
       </c>
       <c r="E538" t="inlineStr">
         <is>
@@ -13798,21 +13798,21 @@
     <row r="539">
       <c r="A539" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:33</t>
         </is>
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D539" t="n">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="E539" t="inlineStr">
         <is>
@@ -13823,21 +13823,21 @@
     <row r="540">
       <c r="A540" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:37</t>
         </is>
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D540" t="n">
-        <v>118</v>
+        <v>68</v>
       </c>
       <c r="E540" t="inlineStr">
         <is>
@@ -13848,21 +13848,21 @@
     <row r="541">
       <c r="A541" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>20:58</t>
+          <t>20:38</t>
         </is>
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D541" t="n">
-        <v>89</v>
+        <v>42</v>
       </c>
       <c r="E541" t="inlineStr">
         <is>
@@ -13873,21 +13873,21 @@
     <row r="542">
       <c r="A542" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>20:58</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D542" t="n">
-        <v>89</v>
+        <v>43</v>
       </c>
       <c r="E542" t="inlineStr">
         <is>
@@ -13903,16 +13903,16 @@
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D543" t="n">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="E543" t="inlineStr">
         <is>
@@ -13928,16 +13928,16 @@
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C544" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D544" t="n">
-        <v>97</v>
+        <v>76</v>
       </c>
       <c r="E544" t="inlineStr">
         <is>
@@ -13948,23 +13948,448 @@
     <row r="545">
       <c r="A545" t="inlineStr">
         <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>20:46</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D545" t="n">
+        <v>50</v>
+      </c>
+      <c r="E545" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
           <t>19:29:54</t>
         </is>
       </c>
-      <c r="B545" t="inlineStr">
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>20:53</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D546" t="n">
+        <v>84</v>
+      </c>
+      <c r="E546" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>18:59:44</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>20:54</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D547" t="n">
+        <v>115</v>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D548" t="n">
+        <v>87</v>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D549" t="n">
+        <v>61</v>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D550" t="n">
+        <v>61</v>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>20:58</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D551" t="n">
+        <v>89</v>
+      </c>
+      <c r="E551" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>20:58</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D552" t="n">
+        <v>89</v>
+      </c>
+      <c r="E552" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>20:59</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D553" t="n">
+        <v>63</v>
+      </c>
+      <c r="E553" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>21:01</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D554" t="n">
+        <v>65</v>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D555" t="n">
+        <v>70</v>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>21:17</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D556" t="n">
+        <v>81</v>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
         <is>
           <t>21:20</t>
         </is>
       </c>
-      <c r="C545" t="inlineStr">
+      <c r="C557" t="inlineStr">
         <is>
           <t>26_HERNANDEZ</t>
         </is>
       </c>
-      <c r="D545" t="n">
+      <c r="D557" t="n">
         <v>111</v>
       </c>
-      <c r="E545" t="inlineStr">
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>21:21</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D558" t="n">
+        <v>85</v>
+      </c>
+      <c r="E558" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D559" t="n">
+        <v>89</v>
+      </c>
+      <c r="E559" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D560" t="n">
+        <v>94</v>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D561" t="n">
+        <v>95</v>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D562" t="n">
+        <v>104</v>
+      </c>
+      <c r="E562" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -13981,7 +14406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13994,14 +14419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:29:54</t>
+          <t>Última actualización: 19:56:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 63</t>
+          <t>Total filas: 64</t>
         </is>
       </c>
     </row>
@@ -15485,7 +15910,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -15499,7 +15924,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>88</v>
+        <v>31</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -15510,7 +15935,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -15524,7 +15949,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -15560,12 +15985,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -15574,7 +15999,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>71</v>
+        <v>43</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -15585,23 +16010,48 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>71</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
           <t>18:59:44</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t>20:54</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D68" t="n">
+      <c r="D69" t="n">
         <v>115</v>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -15618,7 +16068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15631,14 +16081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:29:54</t>
+          <t>Última actualización: 19:56:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 71</t>
+          <t>Total filas: 72</t>
         </is>
       </c>
     </row>
@@ -17297,7 +17747,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -17311,7 +17761,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>89</v>
+        <v>19</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -17347,7 +17797,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -17361,7 +17811,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>95</v>
+        <v>25</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -17397,7 +17847,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -17411,7 +17861,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -17439,6 +17889,31 @@
         <v>85</v>
       </c>
       <c r="E76" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>59</v>
+      </c>
+      <c r="E77" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1780
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E562"/>
+  <dimension ref="A1:E571"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:56:12</t>
+          <t>Última actualización: 20:20:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 557</t>
+          <t>Total filas: 566</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -658,11 +658,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -683,11 +683,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>22</v>
+        <v>113</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>113</v>
+        <v>40</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3583,11 +3583,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4248,7 +4248,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4258,11 +4258,11 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5208,11 +5208,11 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5233,11 +5233,11 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>86X44_EST CHICA-ESC AGRARIA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5383,11 +5383,11 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>86X44_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5458,11 +5458,11 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5483,11 +5483,11 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6908,7 +6908,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7158,11 +7158,11 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,7 +7173,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -7183,11 +7183,11 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7208,7 +7208,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D275" t="n">
@@ -7483,7 +7483,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D286" t="n">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D287" t="n">
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>5</v>
+        <v>62</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D306" t="n">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8258,7 +8258,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D317" t="n">
@@ -8283,7 +8283,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D318" t="n">
@@ -8323,7 +8323,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -8333,11 +8333,11 @@
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -8358,11 +8358,11 @@
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8508,7 +8508,7 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D327" t="n">
@@ -8533,7 +8533,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D328" t="n">
@@ -8683,7 +8683,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D334" t="n">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -9298,7 +9298,7 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
@@ -9308,11 +9308,11 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -9333,7 +9333,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D360" t="n">
@@ -9358,7 +9358,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -9373,7 +9373,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -9383,11 +9383,11 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -9408,7 +9408,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D363" t="n">
@@ -9433,7 +9433,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D364" t="n">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D365" t="n">
@@ -9533,7 +9533,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D368" t="n">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D369" t="n">
@@ -9883,7 +9883,7 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D382" t="n">
@@ -9908,7 +9908,7 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D383" t="n">
@@ -10023,7 +10023,7 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
@@ -10033,11 +10033,11 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>45</v>
+        <v>104</v>
       </c>
       <c r="E388" t="inlineStr">
         <is>
@@ -10048,7 +10048,7 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
@@ -10058,11 +10058,11 @@
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>104</v>
+        <v>45</v>
       </c>
       <c r="E389" t="inlineStr">
         <is>
@@ -10273,7 +10273,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
@@ -10283,11 +10283,11 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E398" t="inlineStr">
         <is>
@@ -10323,7 +10323,7 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
@@ -10333,11 +10333,11 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D400" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E400" t="inlineStr">
         <is>
@@ -10958,7 +10958,7 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D425" t="n">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D426" t="n">
@@ -11048,7 +11048,7 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
@@ -11058,11 +11058,11 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D429" t="n">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="E429" t="inlineStr">
         <is>
@@ -11073,7 +11073,7 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
@@ -11083,11 +11083,11 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D430" t="n">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="E430" t="inlineStr">
         <is>
@@ -11098,7 +11098,7 @@
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
@@ -11108,11 +11108,11 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D431" t="n">
-        <v>112</v>
+        <v>54</v>
       </c>
       <c r="E431" t="inlineStr">
         <is>
@@ -11123,7 +11123,7 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
@@ -11133,11 +11133,11 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D432" t="n">
-        <v>54</v>
+        <v>112</v>
       </c>
       <c r="E432" t="inlineStr">
         <is>
@@ -11198,7 +11198,7 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
@@ -11208,11 +11208,11 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D435" t="n">
-        <v>58</v>
+        <v>116</v>
       </c>
       <c r="E435" t="inlineStr">
         <is>
@@ -11223,7 +11223,7 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
@@ -11233,11 +11233,11 @@
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D436" t="n">
-        <v>12</v>
+        <v>58</v>
       </c>
       <c r="E436" t="inlineStr">
         <is>
@@ -11248,7 +11248,7 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
@@ -11258,11 +11258,11 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D437" t="n">
-        <v>116</v>
+        <v>12</v>
       </c>
       <c r="E437" t="inlineStr">
         <is>
@@ -11283,7 +11283,7 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D438" t="n">
@@ -11308,7 +11308,7 @@
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D439" t="n">
@@ -11633,7 +11633,7 @@
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D452" t="n">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D453" t="n">
@@ -11683,7 +11683,7 @@
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D454" t="n">
@@ -11708,7 +11708,7 @@
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D455" t="n">
@@ -12473,7 +12473,7 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
@@ -12483,11 +12483,11 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D486" t="n">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="E486" t="inlineStr">
         <is>
@@ -12498,7 +12498,7 @@
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
@@ -12508,11 +12508,11 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D487" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="E487" t="inlineStr">
         <is>
@@ -12523,7 +12523,7 @@
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
@@ -12533,11 +12533,11 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D488" t="n">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="E488" t="inlineStr">
         <is>
@@ -12548,7 +12548,7 @@
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B489" t="inlineStr">
@@ -12558,11 +12558,11 @@
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D489" t="n">
-        <v>94</v>
+        <v>22</v>
       </c>
       <c r="E489" t="inlineStr">
         <is>
@@ -12573,7 +12573,7 @@
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B490" t="inlineStr">
@@ -12583,11 +12583,11 @@
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D490" t="n">
-        <v>22</v>
+        <v>94</v>
       </c>
       <c r="E490" t="inlineStr">
         <is>
@@ -13198,7 +13198,7 @@
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B515" t="inlineStr">
@@ -13208,11 +13208,11 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D515" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="E515" t="inlineStr">
         <is>
@@ -13223,7 +13223,7 @@
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B516" t="inlineStr">
@@ -13233,11 +13233,11 @@
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D516" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="E516" t="inlineStr">
         <is>
@@ -13323,7 +13323,7 @@
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B520" t="inlineStr">
@@ -13333,11 +13333,11 @@
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D520" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="E520" t="inlineStr">
         <is>
@@ -13348,7 +13348,7 @@
     <row r="521">
       <c r="A521" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B521" t="inlineStr">
@@ -13358,11 +13358,11 @@
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D521" t="n">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="E521" t="inlineStr">
         <is>
@@ -13598,7 +13598,7 @@
     <row r="531">
       <c r="A531" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B531" t="inlineStr">
@@ -13608,11 +13608,11 @@
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D531" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="E531" t="inlineStr">
         <is>
@@ -13623,12 +13623,12 @@
     <row r="532">
       <c r="A532" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>20:21</t>
+          <t>20:20</t>
         </is>
       </c>
       <c r="C532" t="inlineStr">
@@ -13637,7 +13637,7 @@
         </is>
       </c>
       <c r="D532" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E532" t="inlineStr">
         <is>
@@ -13648,7 +13648,7 @@
     <row r="533">
       <c r="A533" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B533" t="inlineStr">
@@ -13658,11 +13658,11 @@
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D533" t="n">
-        <v>95</v>
+        <v>25</v>
       </c>
       <c r="E533" t="inlineStr">
         <is>
@@ -13673,21 +13673,21 @@
     <row r="534">
       <c r="A534" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B534" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:21</t>
         </is>
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D534" t="n">
-        <v>27</v>
+        <v>95</v>
       </c>
       <c r="E534" t="inlineStr">
         <is>
@@ -13698,21 +13698,21 @@
     <row r="535">
       <c r="A535" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B535" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>20:21</t>
         </is>
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D535" t="n">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="E535" t="inlineStr">
         <is>
@@ -13723,21 +13723,21 @@
     <row r="536">
       <c r="A536" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B536" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C536" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D536" t="n">
-        <v>31</v>
+        <v>3</v>
       </c>
       <c r="E536" t="inlineStr">
         <is>
@@ -13748,21 +13748,21 @@
     <row r="537">
       <c r="A537" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>20:29</t>
+          <t>20:26</t>
         </is>
       </c>
       <c r="C537" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D537" t="n">
-        <v>90</v>
+        <v>57</v>
       </c>
       <c r="E537" t="inlineStr">
         <is>
@@ -13773,21 +13773,21 @@
     <row r="538">
       <c r="A538" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:27</t>
         </is>
       </c>
       <c r="C538" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D538" t="n">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="E538" t="inlineStr">
         <is>
@@ -13798,21 +13798,21 @@
     <row r="539">
       <c r="A539" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>20:33</t>
+          <t>20:29</t>
         </is>
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D539" t="n">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="E539" t="inlineStr">
         <is>
@@ -13823,21 +13823,21 @@
     <row r="540">
       <c r="A540" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>20:37</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D540" t="n">
-        <v>68</v>
+        <v>12</v>
       </c>
       <c r="E540" t="inlineStr">
         <is>
@@ -13848,21 +13848,21 @@
     <row r="541">
       <c r="A541" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>20:38</t>
+          <t>20:33</t>
         </is>
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D541" t="n">
-        <v>42</v>
+        <v>107</v>
       </c>
       <c r="E541" t="inlineStr">
         <is>
@@ -13873,21 +13873,21 @@
     <row r="542">
       <c r="A542" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:37</t>
         </is>
       </c>
       <c r="C542" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D542" t="n">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="E542" t="inlineStr">
         <is>
@@ -13898,12 +13898,12 @@
     <row r="543">
       <c r="A543" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:38</t>
         </is>
       </c>
       <c r="C543" t="inlineStr">
@@ -13912,7 +13912,7 @@
         </is>
       </c>
       <c r="D543" t="n">
-        <v>71</v>
+        <v>18</v>
       </c>
       <c r="E543" t="inlineStr">
         <is>
@@ -13923,21 +13923,21 @@
     <row r="544">
       <c r="A544" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:38</t>
         </is>
       </c>
       <c r="C544" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D544" t="n">
-        <v>76</v>
+        <v>18</v>
       </c>
       <c r="E544" t="inlineStr">
         <is>
@@ -13953,16 +13953,16 @@
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>20:46</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C545" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D545" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E545" t="inlineStr">
         <is>
@@ -13978,16 +13978,16 @@
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>20:53</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C546" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D546" t="n">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="E546" t="inlineStr">
         <is>
@@ -13998,21 +13998,21 @@
     <row r="547">
       <c r="A547" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B547" t="inlineStr">
         <is>
-          <t>20:54</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C547" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D547" t="n">
-        <v>115</v>
+        <v>76</v>
       </c>
       <c r="E547" t="inlineStr">
         <is>
@@ -14023,21 +14023,21 @@
     <row r="548">
       <c r="A548" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B548" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:46</t>
         </is>
       </c>
       <c r="C548" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D548" t="n">
-        <v>87</v>
+        <v>26</v>
       </c>
       <c r="E548" t="inlineStr">
         <is>
@@ -14048,21 +14048,21 @@
     <row r="549">
       <c r="A549" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:53</t>
         </is>
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D549" t="n">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="E549" t="inlineStr">
         <is>
@@ -14073,21 +14073,21 @@
     <row r="550">
       <c r="A550" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:54</t>
         </is>
       </c>
       <c r="C550" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D550" t="n">
-        <v>61</v>
+        <v>115</v>
       </c>
       <c r="E550" t="inlineStr">
         <is>
@@ -14103,7 +14103,7 @@
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>20:58</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C551" t="inlineStr">
@@ -14112,7 +14112,7 @@
         </is>
       </c>
       <c r="D551" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E551" t="inlineStr">
         <is>
@@ -14123,21 +14123,21 @@
     <row r="552">
       <c r="A552" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B552" t="inlineStr">
         <is>
-          <t>20:58</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C552" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D552" t="n">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="E552" t="inlineStr">
         <is>
@@ -14148,21 +14148,21 @@
     <row r="553">
       <c r="A553" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>20:59</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C553" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D553" t="n">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="E553" t="inlineStr">
         <is>
@@ -14173,21 +14173,21 @@
     <row r="554">
       <c r="A554" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B554" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C554" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D554" t="n">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="E554" t="inlineStr">
         <is>
@@ -14198,21 +14198,21 @@
     <row r="555">
       <c r="A555" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B555" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C555" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D555" t="n">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="E555" t="inlineStr">
         <is>
@@ -14228,16 +14228,16 @@
       </c>
       <c r="B556" t="inlineStr">
         <is>
-          <t>21:17</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C556" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D556" t="n">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="E556" t="inlineStr">
         <is>
@@ -14248,21 +14248,21 @@
     <row r="557">
       <c r="A557" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>21:20</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C557" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D557" t="n">
-        <v>111</v>
+        <v>39</v>
       </c>
       <c r="E557" t="inlineStr">
         <is>
@@ -14273,21 +14273,21 @@
     <row r="558">
       <c r="A558" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B558" t="inlineStr">
         <is>
-          <t>21:21</t>
+          <t>21:01</t>
         </is>
       </c>
       <c r="C558" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D558" t="n">
-        <v>85</v>
+        <v>41</v>
       </c>
       <c r="E558" t="inlineStr">
         <is>
@@ -14298,21 +14298,21 @@
     <row r="559">
       <c r="A559" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B559" t="inlineStr">
         <is>
-          <t>21:25</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C559" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D559" t="n">
-        <v>89</v>
+        <v>46</v>
       </c>
       <c r="E559" t="inlineStr">
         <is>
@@ -14323,21 +14323,21 @@
     <row r="560">
       <c r="A560" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>21:12</t>
         </is>
       </c>
       <c r="C560" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D560" t="n">
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="E560" t="inlineStr">
         <is>
@@ -14348,21 +14348,21 @@
     <row r="561">
       <c r="A561" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B561" t="inlineStr">
         <is>
-          <t>21:31</t>
+          <t>21:17</t>
         </is>
       </c>
       <c r="C561" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D561" t="n">
-        <v>95</v>
+        <v>57</v>
       </c>
       <c r="E561" t="inlineStr">
         <is>
@@ -14373,23 +14373,248 @@
     <row r="562">
       <c r="A562" t="inlineStr">
         <is>
+          <t>20:20:36</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>21:20</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D562" t="n">
+        <v>60</v>
+      </c>
+      <c r="E562" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
           <t>19:56:12</t>
         </is>
       </c>
-      <c r="B562" t="inlineStr">
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>21:21</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D563" t="n">
+        <v>85</v>
+      </c>
+      <c r="E563" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D564" t="n">
+        <v>89</v>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>20:20:36</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>21:29</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D565" t="n">
+        <v>69</v>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>20:20:36</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D566" t="n">
+        <v>70</v>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>20:20:36</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D567" t="n">
+        <v>71</v>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>19:56:12</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
         <is>
           <t>21:40</t>
         </is>
       </c>
-      <c r="C562" t="inlineStr">
+      <c r="C568" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D562" t="n">
+      <c r="D568" t="n">
         <v>104</v>
       </c>
-      <c r="E562" t="inlineStr">
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>20:20:36</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>21:41</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D569" t="n">
+        <v>81</v>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>20:20:36</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>21:52</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D570" t="n">
+        <v>92</v>
+      </c>
+      <c r="E570" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>20:20:36</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>22:01</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D571" t="n">
+        <v>101</v>
+      </c>
+      <c r="E571" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -14406,7 +14631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14419,14 +14644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:56:12</t>
+          <t>Última actualización: 20:20:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 64</t>
+          <t>Total filas: 65</t>
         </is>
       </c>
     </row>
@@ -15910,7 +16135,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -15924,7 +16149,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -15935,7 +16160,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -15949,7 +16174,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -15985,12 +16210,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:38</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -15999,7 +16224,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -16010,12 +16235,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -16024,7 +16249,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>71</v>
+        <v>43</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -16035,23 +16260,48 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
+          <t>19:29:54</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>71</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
           <t>18:59:44</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t>20:54</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D69" t="n">
+      <c r="D70" t="n">
         <v>115</v>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -16068,7 +16318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16081,14 +16331,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:56:12</t>
+          <t>Última actualización: 20:20:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 72</t>
+          <t>Total filas: 75</t>
         </is>
       </c>
     </row>
@@ -17822,21 +18072,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:22</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>66</v>
+        <v>2</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -17847,12 +18097,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -17861,7 +18111,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -17872,50 +18122,125 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>20:54</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>85</v>
+        <v>40</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t>20:20:36</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>20:54</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>34</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
           <t>19:56:12</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B78" t="inlineStr">
         <is>
           <t>20:55</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D77" t="n">
+      <c r="D78" t="n">
         <v>59</v>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="E78" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>20:20:36</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>98</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>20:20:36</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>115</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1781
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E571"/>
+  <dimension ref="A1:E581"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:20:36</t>
+          <t>Última actualización: 20:48:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 566</t>
+          <t>Total filas: 576</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>18</v>
+        <v>86</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3033,11 +3033,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3358,7 +3358,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>22</v>
+        <v>113</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215D_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215D_EL PATO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D140" t="n">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D141" t="n">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
@@ -3933,7 +3933,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D145" t="n">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D156" t="n">
@@ -4248,7 +4248,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4258,11 +4258,11 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4358,7 +4358,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D161" t="n">
@@ -4383,7 +4383,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D162" t="n">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5458,11 +5458,11 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5483,11 +5483,11 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5633,7 +5633,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D213" t="n">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6883,11 +6883,11 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>10_RUTA 36_ESC 70</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>90</v>
+        <v>4</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6908,7 +6908,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6933,11 +6933,11 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_RUTA 36_ESC 70</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>4</v>
+        <v>90</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6983,7 +6983,7 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D266" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D267" t="n">
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7173,7 +7173,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -7183,11 +7183,11 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,7 +7198,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -7208,11 +7208,11 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7558,7 +7558,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D289" t="n">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D305" t="n">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8258,7 +8258,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D317" t="n">
@@ -8283,7 +8283,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D318" t="n">
@@ -8433,7 +8433,7 @@
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D324" t="n">
@@ -8458,7 +8458,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D325" t="n">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D330" t="n">
@@ -8683,7 +8683,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D334" t="n">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -9298,7 +9298,7 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
@@ -9308,11 +9308,11 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -9358,7 +9358,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -9373,7 +9373,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -9383,11 +9383,11 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -9433,7 +9433,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D364" t="n">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D365" t="n">
@@ -9883,7 +9883,7 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D382" t="n">
@@ -9908,7 +9908,7 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D383" t="n">
@@ -10083,7 +10083,7 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D390" t="n">
@@ -10108,7 +10108,7 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D391" t="n">
@@ -10273,7 +10273,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
@@ -10283,11 +10283,11 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E398" t="inlineStr">
         <is>
@@ -10298,7 +10298,7 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
@@ -10308,11 +10308,11 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D399" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E399" t="inlineStr">
         <is>
@@ -10333,7 +10333,7 @@
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D400" t="n">
@@ -10398,7 +10398,7 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
@@ -10408,11 +10408,11 @@
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D403" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="E403" t="inlineStr">
         <is>
@@ -10423,7 +10423,7 @@
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
@@ -10433,11 +10433,11 @@
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D404" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E404" t="inlineStr">
         <is>
@@ -10583,7 +10583,7 @@
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D410" t="n">
@@ -10633,7 +10633,7 @@
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D412" t="n">
@@ -10798,7 +10798,7 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
@@ -10808,11 +10808,11 @@
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D419" t="n">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="E419" t="inlineStr">
         <is>
@@ -10823,7 +10823,7 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
@@ -10833,11 +10833,11 @@
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D420" t="n">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E420" t="inlineStr">
         <is>
@@ -10958,7 +10958,7 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D425" t="n">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D426" t="n">
@@ -11008,7 +11008,7 @@
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D427" t="n">
@@ -11033,7 +11033,7 @@
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D428" t="n">
@@ -11098,7 +11098,7 @@
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
@@ -11108,11 +11108,11 @@
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D431" t="n">
-        <v>54</v>
+        <v>112</v>
       </c>
       <c r="E431" t="inlineStr">
         <is>
@@ -11123,7 +11123,7 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
@@ -11133,11 +11133,11 @@
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D432" t="n">
-        <v>112</v>
+        <v>54</v>
       </c>
       <c r="E432" t="inlineStr">
         <is>
@@ -11198,7 +11198,7 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
@@ -11208,11 +11208,11 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D435" t="n">
-        <v>116</v>
+        <v>58</v>
       </c>
       <c r="E435" t="inlineStr">
         <is>
@@ -11223,7 +11223,7 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
@@ -11233,11 +11233,11 @@
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D436" t="n">
-        <v>58</v>
+        <v>116</v>
       </c>
       <c r="E436" t="inlineStr">
         <is>
@@ -11283,7 +11283,7 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D438" t="n">
@@ -11308,7 +11308,7 @@
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D439" t="n">
@@ -11583,7 +11583,7 @@
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D450" t="n">
@@ -11608,7 +11608,7 @@
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D451" t="n">
@@ -11633,7 +11633,7 @@
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D452" t="n">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D453" t="n">
@@ -11683,7 +11683,7 @@
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D454" t="n">
@@ -11708,7 +11708,7 @@
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D455" t="n">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D482" t="n">
@@ -12408,7 +12408,7 @@
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D483" t="n">
@@ -12423,7 +12423,7 @@
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
@@ -12433,11 +12433,11 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D484" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="E484" t="inlineStr">
         <is>
@@ -12448,7 +12448,7 @@
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B485" t="inlineStr">
@@ -12458,11 +12458,11 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D485" t="n">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="E485" t="inlineStr">
         <is>
@@ -12473,7 +12473,7 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
@@ -12483,11 +12483,11 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D486" t="n">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="E486" t="inlineStr">
         <is>
@@ -12523,7 +12523,7 @@
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
@@ -12533,11 +12533,11 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D488" t="n">
-        <v>64</v>
+        <v>20</v>
       </c>
       <c r="E488" t="inlineStr">
         <is>
@@ -12623,7 +12623,7 @@
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B492" t="inlineStr">
@@ -12633,11 +12633,11 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D492" t="n">
-        <v>25</v>
+        <v>97</v>
       </c>
       <c r="E492" t="inlineStr">
         <is>
@@ -12648,7 +12648,7 @@
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B493" t="inlineStr">
@@ -12658,11 +12658,11 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D493" t="n">
-        <v>97</v>
+        <v>25</v>
       </c>
       <c r="E493" t="inlineStr">
         <is>
@@ -12923,7 +12923,7 @@
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B504" t="inlineStr">
@@ -12933,11 +12933,11 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D504" t="n">
-        <v>14</v>
+        <v>88</v>
       </c>
       <c r="E504" t="inlineStr">
         <is>
@@ -12948,7 +12948,7 @@
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B505" t="inlineStr">
@@ -12958,11 +12958,11 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D505" t="n">
-        <v>88</v>
+        <v>14</v>
       </c>
       <c r="E505" t="inlineStr">
         <is>
@@ -13198,7 +13198,7 @@
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B515" t="inlineStr">
@@ -13208,11 +13208,11 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D515" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="E515" t="inlineStr">
         <is>
@@ -13223,7 +13223,7 @@
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B516" t="inlineStr">
@@ -13233,11 +13233,11 @@
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D516" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="E516" t="inlineStr">
         <is>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D531" t="n">
@@ -13633,7 +13633,7 @@
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D532" t="n">
@@ -13648,7 +13648,7 @@
     <row r="533">
       <c r="A533" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B533" t="inlineStr">
@@ -13658,11 +13658,11 @@
       </c>
       <c r="C533" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D533" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E533" t="inlineStr">
         <is>
@@ -13698,7 +13698,7 @@
     <row r="535">
       <c r="A535" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B535" t="inlineStr">
@@ -13708,11 +13708,11 @@
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D535" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="E535" t="inlineStr">
         <is>
@@ -13908,7 +13908,7 @@
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D543" t="n">
@@ -13933,7 +13933,7 @@
       </c>
       <c r="C544" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D544" t="n">
@@ -14048,21 +14048,21 @@
     <row r="549">
       <c r="A549" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>20:53</t>
+          <t>20:49</t>
         </is>
       </c>
       <c r="C549" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D549" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E549" t="inlineStr">
         <is>
@@ -14073,12 +14073,12 @@
     <row r="550">
       <c r="A550" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>20:54</t>
+          <t>20:49</t>
         </is>
       </c>
       <c r="C550" t="inlineStr">
@@ -14087,7 +14087,7 @@
         </is>
       </c>
       <c r="D550" t="n">
-        <v>115</v>
+        <v>1</v>
       </c>
       <c r="E550" t="inlineStr">
         <is>
@@ -14103,16 +14103,16 @@
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:53</t>
         </is>
       </c>
       <c r="C551" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D551" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E551" t="inlineStr">
         <is>
@@ -14123,21 +14123,21 @@
     <row r="552">
       <c r="A552" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B552" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:54</t>
         </is>
       </c>
       <c r="C552" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D552" t="n">
-        <v>61</v>
+        <v>115</v>
       </c>
       <c r="E552" t="inlineStr">
         <is>
@@ -14148,21 +14148,21 @@
     <row r="553">
       <c r="A553" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B553" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C553" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D553" t="n">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="E553" t="inlineStr">
         <is>
@@ -14173,12 +14173,12 @@
     <row r="554">
       <c r="A554" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B554" t="inlineStr">
         <is>
-          <t>20:58</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C554" t="inlineStr">
@@ -14187,7 +14187,7 @@
         </is>
       </c>
       <c r="D554" t="n">
-        <v>89</v>
+        <v>8</v>
       </c>
       <c r="E554" t="inlineStr">
         <is>
@@ -14203,16 +14203,16 @@
       </c>
       <c r="B555" t="inlineStr">
         <is>
-          <t>20:58</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C555" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D555" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E555" t="inlineStr">
         <is>
@@ -14228,16 +14228,16 @@
       </c>
       <c r="B556" t="inlineStr">
         <is>
-          <t>20:59</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C556" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D556" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E556" t="inlineStr">
         <is>
@@ -14248,21 +14248,21 @@
     <row r="557">
       <c r="A557" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>20:59</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C557" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D557" t="n">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="E557" t="inlineStr">
         <is>
@@ -14273,21 +14273,21 @@
     <row r="558">
       <c r="A558" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B558" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C558" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D558" t="n">
-        <v>41</v>
+        <v>89</v>
       </c>
       <c r="E558" t="inlineStr">
         <is>
@@ -14303,16 +14303,16 @@
       </c>
       <c r="B559" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C559" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D559" t="n">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="E559" t="inlineStr">
         <is>
@@ -14323,21 +14323,21 @@
     <row r="560">
       <c r="A560" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>21:12</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C560" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D560" t="n">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="E560" t="inlineStr">
         <is>
@@ -14348,21 +14348,21 @@
     <row r="561">
       <c r="A561" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B561" t="inlineStr">
         <is>
-          <t>21:17</t>
+          <t>21:01</t>
         </is>
       </c>
       <c r="C561" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D561" t="n">
-        <v>57</v>
+        <v>13</v>
       </c>
       <c r="E561" t="inlineStr">
         <is>
@@ -14373,21 +14373,21 @@
     <row r="562">
       <c r="A562" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>21:20</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C562" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D562" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="E562" t="inlineStr">
         <is>
@@ -14398,21 +14398,21 @@
     <row r="563">
       <c r="A563" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B563" t="inlineStr">
         <is>
-          <t>21:21</t>
+          <t>21:12</t>
         </is>
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D563" t="n">
-        <v>85</v>
+        <v>24</v>
       </c>
       <c r="E563" t="inlineStr">
         <is>
@@ -14423,21 +14423,21 @@
     <row r="564">
       <c r="A564" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B564" t="inlineStr">
         <is>
-          <t>21:25</t>
+          <t>21:16</t>
         </is>
       </c>
       <c r="C564" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D564" t="n">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="E564" t="inlineStr">
         <is>
@@ -14453,16 +14453,16 @@
       </c>
       <c r="B565" t="inlineStr">
         <is>
-          <t>21:29</t>
+          <t>21:17</t>
         </is>
       </c>
       <c r="C565" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D565" t="n">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="E565" t="inlineStr">
         <is>
@@ -14473,21 +14473,21 @@
     <row r="566">
       <c r="A566" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>21:20</t>
         </is>
       </c>
       <c r="C566" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D566" t="n">
-        <v>70</v>
+        <v>32</v>
       </c>
       <c r="E566" t="inlineStr">
         <is>
@@ -14498,21 +14498,21 @@
     <row r="567">
       <c r="A567" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>21:31</t>
+          <t>21:21</t>
         </is>
       </c>
       <c r="C567" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D567" t="n">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="E567" t="inlineStr">
         <is>
@@ -14528,16 +14528,16 @@
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>21:40</t>
+          <t>21:25</t>
         </is>
       </c>
       <c r="C568" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D568" t="n">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="E568" t="inlineStr">
         <is>
@@ -14548,21 +14548,21 @@
     <row r="569">
       <c r="A569" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B569" t="inlineStr">
         <is>
-          <t>21:41</t>
+          <t>21:29</t>
         </is>
       </c>
       <c r="C569" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D569" t="n">
-        <v>81</v>
+        <v>41</v>
       </c>
       <c r="E569" t="inlineStr">
         <is>
@@ -14573,21 +14573,21 @@
     <row r="570">
       <c r="A570" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>21:52</t>
+          <t>21:29</t>
         </is>
       </c>
       <c r="C570" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D570" t="n">
-        <v>92</v>
+        <v>41</v>
       </c>
       <c r="E570" t="inlineStr">
         <is>
@@ -14603,18 +14603,268 @@
       </c>
       <c r="B571" t="inlineStr">
         <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D571" t="n">
+        <v>70</v>
+      </c>
+      <c r="E571" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>20:48:48</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D572" t="n">
+        <v>43</v>
+      </c>
+      <c r="E572" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>20:48:48</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D573" t="n">
+        <v>52</v>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>20:20:36</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>21:41</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D574" t="n">
+        <v>81</v>
+      </c>
+      <c r="E574" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>20:48:48</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>21:52</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D575" t="n">
+        <v>64</v>
+      </c>
+      <c r="E575" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>20:48:48</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D576" t="n">
+        <v>71</v>
+      </c>
+      <c r="E576" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>20:48:48</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
           <t>22:01</t>
         </is>
       </c>
-      <c r="C571" t="inlineStr">
+      <c r="C577" t="inlineStr">
         <is>
           <t>15_P INDUSTRIAL</t>
         </is>
       </c>
-      <c r="D571" t="n">
-        <v>101</v>
-      </c>
-      <c r="E571" t="inlineStr">
+      <c r="D577" t="n">
+        <v>73</v>
+      </c>
+      <c r="E577" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>20:48:48</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>22:16</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D578" t="n">
+        <v>88</v>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>20:48:48</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>22:20</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D579" t="n">
+        <v>92</v>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>20:48:48</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>22:31</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D580" t="n">
+        <v>103</v>
+      </c>
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>20:48:48</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>22:41</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D581" t="n">
+        <v>113</v>
+      </c>
+      <c r="E581" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -14631,7 +14881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14644,14 +14894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:20:36</t>
+          <t>Última actualización: 20:48:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 65</t>
+          <t>Total filas: 66</t>
         </is>
       </c>
     </row>
@@ -16285,23 +16535,48 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
+          <t>20:48:48</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>20:49</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
           <t>18:59:44</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t>20:54</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C71" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D70" t="n">
+      <c r="D71" t="n">
         <v>115</v>
       </c>
-      <c r="E70" t="inlineStr">
+      <c r="E71" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -16318,7 +16593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16331,14 +16606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:20:36</t>
+          <t>Última actualización: 20:48:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 75</t>
+          <t>Total filas: 77</t>
         </is>
       </c>
     </row>
@@ -18147,7 +18422,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -18161,7 +18436,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -18197,7 +18472,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -18211,7 +18486,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>98</v>
+        <v>70</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -18222,25 +18497,75 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
+          <t>20:48:48</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>22:13</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>85</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
           <t>20:20:36</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>22:15</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D80" t="n">
+      <c r="D81" t="n">
         <v>115</v>
       </c>
-      <c r="E80" t="inlineStr">
+      <c r="E81" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>20:48:48</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>22:25</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>97</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1782
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-20.xlsx
+++ b/data/horarios-141-2026-03-20.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E581"/>
+  <dimension ref="A1:E591"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:48:48</t>
+          <t>Última actualización: 21:01:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 576</t>
+          <t>Total filas: 586</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:52:36</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -658,11 +658,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:52:36</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -683,11 +683,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:28:28</t>
+          <t>04:09:32</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -733,11 +733,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,7 +748,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:09:32</t>
+          <t>05:28:28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -758,11 +758,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>83</v>
+        <v>4</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>06:05:16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:05:16</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1823,7 +1823,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1833,11 +1833,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>06:55:38</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>06:55:38</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2533,11 +2533,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,7 +2823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2833,11 +2833,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D114" t="n">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:03:22</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3358,7 +3358,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>08:03:22</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>07:27:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>08:40:05</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>08:40:05</t>
+          <t>07:27:56</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D152" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4248,7 +4248,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>08:58:21</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4258,11 +4258,11 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>08:58:21</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>17/64_OLMOS POR 520</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17/64_OLMOS POR 520</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>62</v>
+        <v>2</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4858,7 +4858,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>09:53:56</t>
+          <t>10:53:20</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5458,11 +5458,11 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>10:53:20</t>
+          <t>09:53:56</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5483,11 +5483,11 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D209" t="n">
@@ -5583,7 +5583,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ESC 3-ESC 61-ETCHEVERRY</t>
         </is>
       </c>
       <c r="D211" t="n">
@@ -5908,7 +5908,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D223" t="n">
@@ -5933,7 +5933,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D240" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -6383,7 +6383,7 @@
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D242" t="n">
@@ -6408,7 +6408,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D243" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6623,7 +6623,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6633,11 +6633,11 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6658,11 +6658,11 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>12</v>
+        <v>61</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6808,7 +6808,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D262" t="n">
@@ -6908,7 +6908,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -6948,7 +6948,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>11:35:43</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -6958,11 +6958,11 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>6</v>
+        <v>92</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,7 +6973,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>11:35:43</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -6983,11 +6983,11 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>92</v>
+        <v>6</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -7008,7 +7008,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D267" t="n">
@@ -7023,7 +7023,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -7033,11 +7033,11 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,7 +7048,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -7058,11 +7058,11 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7173,7 +7173,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>12:24:25</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -7183,11 +7183,11 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,7 +7198,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>12:24:25</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -7208,11 +7208,11 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7483,7 +7483,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D286" t="n">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D287" t="n">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D289" t="n">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>13:58:21</t>
+          <t>13:01:41</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17_179 Y 38</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>5</v>
+        <v>62</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,7 +7723,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>13:01:41</t>
+          <t>13:58:21</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7733,11 +7733,11 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>17_179 Y 38</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>62</v>
+        <v>5</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7958,7 +7958,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D305" t="n">
@@ -7983,7 +7983,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D306" t="n">
@@ -8258,7 +8258,7 @@
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D317" t="n">
@@ -8283,7 +8283,7 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D318" t="n">
@@ -8483,7 +8483,7 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D326" t="n">
@@ -8533,7 +8533,7 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D328" t="n">
@@ -8683,7 +8683,7 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D334" t="n">
@@ -8708,7 +8708,7 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D335" t="n">
@@ -9048,7 +9048,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -9058,11 +9058,11 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,7 +9073,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -9083,11 +9083,11 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9308,7 +9308,7 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D359" t="n">
@@ -9333,7 +9333,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>86_EST CHICA-ESC AGRARIA</t>
         </is>
       </c>
       <c r="D360" t="n">
@@ -9348,7 +9348,7 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>14:33:32</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
@@ -9358,11 +9358,11 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>86_EST CHICA-ESC AGRARIA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -9373,7 +9373,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>14:33:32</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -9383,11 +9383,11 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -9408,7 +9408,7 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D363" t="n">
@@ -9458,7 +9458,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D365" t="n">
@@ -9533,7 +9533,7 @@
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D368" t="n">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D369" t="n">
@@ -9883,7 +9883,7 @@
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D382" t="n">
@@ -9908,7 +9908,7 @@
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D383" t="n">
@@ -9923,7 +9923,7 @@
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>16:03:30</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
@@ -9933,11 +9933,11 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="E384" t="inlineStr">
         <is>
@@ -9948,7 +9948,7 @@
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>16:03:30</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
@@ -9958,11 +9958,11 @@
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="E385" t="inlineStr">
         <is>
@@ -10083,7 +10083,7 @@
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D390" t="n">
@@ -10108,7 +10108,7 @@
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D391" t="n">
@@ -10123,7 +10123,7 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>15:04:05</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
@@ -10133,11 +10133,11 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>109</v>
+        <v>11</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -10148,7 +10148,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>15:04:05</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
@@ -10158,11 +10158,11 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>11</v>
+        <v>109</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -10273,7 +10273,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
@@ -10283,11 +10283,11 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E398" t="inlineStr">
         <is>
@@ -10298,7 +10298,7 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
@@ -10308,11 +10308,11 @@
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D399" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E399" t="inlineStr">
         <is>
@@ -10958,7 +10958,7 @@
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D425" t="n">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D426" t="n">
@@ -11048,7 +11048,7 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>16:42:24</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
@@ -11058,11 +11058,11 @@
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_155 Y 38-B MALVINAS</t>
         </is>
       </c>
       <c r="D429" t="n">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="E429" t="inlineStr">
         <is>
@@ -11073,7 +11073,7 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>16:42:24</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
@@ -11083,11 +11083,11 @@
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>26_155 Y 38-B MALVINAS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D430" t="n">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="E430" t="inlineStr">
         <is>
@@ -11198,7 +11198,7 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
@@ -11208,11 +11208,11 @@
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D435" t="n">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="E435" t="inlineStr">
         <is>
@@ -11248,7 +11248,7 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
@@ -11258,11 +11258,11 @@
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D437" t="n">
-        <v>12</v>
+        <v>58</v>
       </c>
       <c r="E437" t="inlineStr">
         <is>
@@ -11548,7 +11548,7 @@
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>17:01:59</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
@@ -11558,11 +11558,11 @@
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D449" t="n">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="E449" t="inlineStr">
         <is>
@@ -11573,7 +11573,7 @@
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>17:01:59</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
@@ -11583,11 +11583,11 @@
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D450" t="n">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="E450" t="inlineStr">
         <is>
@@ -11633,7 +11633,7 @@
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D452" t="n">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D453" t="n">
@@ -11683,7 +11683,7 @@
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D454" t="n">
@@ -11708,7 +11708,7 @@
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D455" t="n">
@@ -12423,7 +12423,7 @@
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
@@ -12433,11 +12433,11 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D484" t="n">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="E484" t="inlineStr">
         <is>
@@ -12448,7 +12448,7 @@
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B485" t="inlineStr">
@@ -12458,11 +12458,11 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D485" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="E485" t="inlineStr">
         <is>
@@ -12473,7 +12473,7 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
@@ -12483,11 +12483,11 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D486" t="n">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="E486" t="inlineStr">
         <is>
@@ -12498,7 +12498,7 @@
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
@@ -12508,11 +12508,11 @@
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D487" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="E487" t="inlineStr">
         <is>
@@ -12523,7 +12523,7 @@
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
@@ -12533,11 +12533,11 @@
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D488" t="n">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="E488" t="inlineStr">
         <is>
@@ -12623,7 +12623,7 @@
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>17:47:44</t>
+          <t>18:59:44</t>
         </is>
       </c>
       <c r="B492" t="inlineStr">
@@ -12633,11 +12633,11 @@
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D492" t="n">
-        <v>97</v>
+        <v>25</v>
       </c>
       <c r="E492" t="inlineStr">
         <is>
@@ -12648,7 +12648,7 @@
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>18:59:44</t>
+          <t>17:47:44</t>
         </is>
       </c>
       <c r="B493" t="inlineStr">
@@ -12658,11 +12658,11 @@
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D493" t="n">
-        <v>25</v>
+        <v>97</v>
       </c>
       <c r="E493" t="inlineStr">
         <is>
@@ -12808,7 +12808,7 @@
       </c>
       <c r="C499" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D499" t="n">
@@ -12833,7 +12833,7 @@
       </c>
       <c r="C500" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D500" t="n">
@@ -12923,7 +12923,7 @@
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B504" t="inlineStr">
@@ -12933,11 +12933,11 @@
       </c>
       <c r="C504" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D504" t="n">
-        <v>88</v>
+        <v>14</v>
       </c>
       <c r="E504" t="inlineStr">
         <is>
@@ -12948,7 +12948,7 @@
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B505" t="inlineStr">
@@ -12958,11 +12958,11 @@
       </c>
       <c r="C505" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D505" t="n">
-        <v>14</v>
+        <v>88</v>
       </c>
       <c r="E505" t="inlineStr">
         <is>
@@ -13048,7 +13048,7 @@
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>18:15:10</t>
         </is>
       </c>
       <c r="B509" t="inlineStr">
@@ -13058,11 +13058,11 @@
       </c>
       <c r="C509" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D509" t="n">
-        <v>22</v>
+        <v>96</v>
       </c>
       <c r="E509" t="inlineStr">
         <is>
@@ -13073,7 +13073,7 @@
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>18:15:10</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B510" t="inlineStr">
@@ -13083,11 +13083,11 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D510" t="n">
-        <v>96</v>
+        <v>22</v>
       </c>
       <c r="E510" t="inlineStr">
         <is>
@@ -13148,7 +13148,7 @@
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B513" t="inlineStr">
@@ -13158,11 +13158,11 @@
       </c>
       <c r="C513" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D513" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E513" t="inlineStr">
         <is>
@@ -13173,7 +13173,7 @@
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B514" t="inlineStr">
@@ -13183,11 +13183,11 @@
       </c>
       <c r="C514" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D514" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="E514" t="inlineStr">
         <is>
@@ -13198,7 +13198,7 @@
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>19:29:54</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B515" t="inlineStr">
@@ -13208,11 +13208,11 @@
       </c>
       <c r="C515" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D515" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="E515" t="inlineStr">
         <is>
@@ -13223,7 +13223,7 @@
     <row r="516">
       <c r="A516" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>19:29:54</t>
         </is>
       </c>
       <c r="B516" t="inlineStr">
@@ -13233,11 +13233,11 @@
       </c>
       <c r="C516" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D516" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="E516" t="inlineStr">
         <is>
@@ -13323,7 +13323,7 @@
     <row r="520">
       <c r="A520" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B520" t="inlineStr">
@@ -13333,11 +13333,11 @@
       </c>
       <c r="C520" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D520" t="n">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="E520" t="inlineStr">
         <is>
@@ -13348,7 +13348,7 @@
     <row r="521">
       <c r="A521" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B521" t="inlineStr">
@@ -13358,11 +13358,11 @@
       </c>
       <c r="C521" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D521" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="E521" t="inlineStr">
         <is>
@@ -13523,7 +13523,7 @@
     <row r="528">
       <c r="A528" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B528" t="inlineStr">
@@ -13533,11 +13533,11 @@
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_P MOR-167 Y 521</t>
         </is>
       </c>
       <c r="D528" t="n">
-        <v>21</v>
+        <v>91</v>
       </c>
       <c r="E528" t="inlineStr">
         <is>
@@ -13548,7 +13548,7 @@
     <row r="529">
       <c r="A529" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B529" t="inlineStr">
@@ -13558,11 +13558,11 @@
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>16_P MOR-167 Y 521</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D529" t="n">
-        <v>91</v>
+        <v>21</v>
       </c>
       <c r="E529" t="inlineStr">
         <is>
@@ -13608,7 +13608,7 @@
       </c>
       <c r="C531" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D531" t="n">
@@ -13633,7 +13633,7 @@
       </c>
       <c r="C532" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D532" t="n">
@@ -13673,7 +13673,7 @@
     <row r="534">
       <c r="A534" t="inlineStr">
         <is>
-          <t>18:46:01</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B534" t="inlineStr">
@@ -13683,11 +13683,11 @@
       </c>
       <c r="C534" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D534" t="n">
-        <v>95</v>
+        <v>25</v>
       </c>
       <c r="E534" t="inlineStr">
         <is>
@@ -13698,7 +13698,7 @@
     <row r="535">
       <c r="A535" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>18:46:01</t>
         </is>
       </c>
       <c r="B535" t="inlineStr">
@@ -13708,11 +13708,11 @@
       </c>
       <c r="C535" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D535" t="n">
-        <v>25</v>
+        <v>95</v>
       </c>
       <c r="E535" t="inlineStr">
         <is>
@@ -13908,7 +13908,7 @@
       </c>
       <c r="C543" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D543" t="n">
@@ -13933,7 +13933,7 @@
       </c>
       <c r="C544" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D544" t="n">
@@ -14298,7 +14298,7 @@
     <row r="559">
       <c r="A559" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B559" t="inlineStr">
@@ -14308,11 +14308,11 @@
       </c>
       <c r="C559" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D559" t="n">
-        <v>39</v>
+        <v>63</v>
       </c>
       <c r="E559" t="inlineStr">
         <is>
@@ -14323,7 +14323,7 @@
     <row r="560">
       <c r="A560" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B560" t="inlineStr">
@@ -14333,11 +14333,11 @@
       </c>
       <c r="C560" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D560" t="n">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="E560" t="inlineStr">
         <is>
@@ -14348,7 +14348,7 @@
     <row r="561">
       <c r="A561" t="inlineStr">
         <is>
-          <t>20:48:48</t>
+          <t>21:01:13</t>
         </is>
       </c>
       <c r="B561" t="inlineStr">
@@ -14362,7 +14362,7 @@
         </is>
       </c>
       <c r="D561" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E561" t="inlineStr">
         <is>
@@ -14373,21 +14373,21 @@
     <row r="562">
       <c r="A562" t="inlineStr">
         <is>
-          <t>20:48:48</t>
+          <t>21:01:13</t>
         </is>
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C562" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D562" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E562" t="inlineStr">
         <is>
@@ -14398,21 +14398,21 @@
     <row r="563">
       <c r="A563" t="inlineStr">
         <is>
-          <t>20:48:48</t>
+          <t>21:01:13</t>
         </is>
       </c>
       <c r="B563" t="inlineStr">
         <is>
-          <t>21:12</t>
+          <t>21:04</t>
         </is>
       </c>
       <c r="C563" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D563" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="E563" t="inlineStr">
         <is>
@@ -14428,16 +14428,16 @@
       </c>
       <c r="B564" t="inlineStr">
         <is>
-          <t>21:16</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C564" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D564" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="E564" t="inlineStr">
         <is>
@@ -14448,21 +14448,21 @@
     <row r="565">
       <c r="A565" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B565" t="inlineStr">
         <is>
-          <t>21:17</t>
+          <t>21:12</t>
         </is>
       </c>
       <c r="C565" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D565" t="n">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="E565" t="inlineStr">
         <is>
@@ -14473,21 +14473,21 @@
     <row r="566">
       <c r="A566" t="inlineStr">
         <is>
-          <t>20:48:48</t>
+          <t>21:01:13</t>
         </is>
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t>21:20</t>
+          <t>21:13</t>
         </is>
       </c>
       <c r="C566" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D566" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="E566" t="inlineStr">
         <is>
@@ -14498,21 +14498,21 @@
     <row r="567">
       <c r="A567" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>20:48:48</t>
         </is>
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>21:21</t>
+          <t>21:16</t>
         </is>
       </c>
       <c r="C567" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D567" t="n">
-        <v>85</v>
+        <v>28</v>
       </c>
       <c r="E567" t="inlineStr">
         <is>
@@ -14523,21 +14523,21 @@
     <row r="568">
       <c r="A568" t="inlineStr">
         <is>
-          <t>19:56:12</t>
+          <t>21:01:13</t>
         </is>
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>21:25</t>
+          <t>21:17</t>
         </is>
       </c>
       <c r="C568" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D568" t="n">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="E568" t="inlineStr">
         <is>
@@ -14553,16 +14553,16 @@
       </c>
       <c r="B569" t="inlineStr">
         <is>
-          <t>21:29</t>
+          <t>21:20</t>
         </is>
       </c>
       <c r="C569" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D569" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="E569" t="inlineStr">
         <is>
@@ -14573,21 +14573,21 @@
     <row r="570">
       <c r="A570" t="inlineStr">
         <is>
-          <t>20:48:48</t>
+          <t>21:01:13</t>
         </is>
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>21:29</t>
+          <t>21:21</t>
         </is>
       </c>
       <c r="C570" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D570" t="n">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="E570" t="inlineStr">
         <is>
@@ -14598,21 +14598,21 @@
     <row r="571">
       <c r="A571" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>19:56:12</t>
         </is>
       </c>
       <c r="B571" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>21:25</t>
         </is>
       </c>
       <c r="C571" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D571" t="n">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="E571" t="inlineStr">
         <is>
@@ -14628,16 +14628,16 @@
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>21:31</t>
+          <t>21:29</t>
         </is>
       </c>
       <c r="C572" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D572" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E572" t="inlineStr">
         <is>
@@ -14653,16 +14653,16 @@
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>21:40</t>
+          <t>21:29</t>
         </is>
       </c>
       <c r="C573" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D573" t="n">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E573" t="inlineStr">
         <is>
@@ -14673,21 +14673,21 @@
     <row r="574">
       <c r="A574" t="inlineStr">
         <is>
-          <t>20:20:36</t>
+          <t>21:01:13</t>
         </is>
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>21:41</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C574" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D574" t="n">
-        <v>81</v>
+        <v>29</v>
       </c>
       <c r="E574" t="inlineStr">
         <is>
@@ -14698,21 +14698,21 @@
     <row r="575">
       <c r="A575" t="inlineStr">
         <is>
-          <t>20:48:48</t>
+          <t>21:01:13</t>
         </is>
       </c>
       <c r="B575" t="inlineStr">
         <is>
-          <t>21:52</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C575" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D575" t="n">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="E575" t="inlineStr">
         <is>
@@ -14723,21 +14723,21 @@
     <row r="576">
       <c r="A576" t="inlineStr">
         <is>
-          <t>20:48:48</t>
+          <t>21:01:13</t>
         </is>
       </c>
       <c r="B576" t="inlineStr">
         <is>
-          <t>21:59</t>
+          <t>21:31</t>
         </is>
       </c>
       <c r="C576" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D576" t="n">
-        <v>71</v>
+        <v>30</v>
       </c>
       <c r="E576" t="inlineStr">
         <is>
@@ -14748,21 +14748,21 @@
     <row r="577">
       <c r="A577" t="inlineStr">
         <is>
-          <t>20:48:48</t>
+          <t>21:01:13</t>
         </is>
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>22:01</t>
+          <t>21:40</t>
         </is>
       </c>
       <c r="C577" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D577" t="n">
-        <v>73</v>
+        <v>39</v>
       </c>
       <c r="E577" t="inlineStr">
         <is>
@@ -14773,21 +14773,21 @@
     <row r="578">
       <c r="A578" t="inlineStr">
         <is>
-          <t>20:48:48</t>
+          <t>20:20:36</t>
         </is>
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>22:16</t>
+          <t>21:41</t>
         </is>
       </c>
       <c r="C578" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D578" t="n">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="E578" t="inlineStr">
         <is>
@@ -14798,21 +14798,21 @@
     <row r="579">
       <c r="A579" t="inlineStr">
         <is>
-          <t>20:48:48</t>
+          <t>21:01:13</t>
         </is>
       </c>
       <c r="B579" t="inlineStr">
         <is>
-          <t>22:20</t>
+          <t>21:52</t>
         </is>
       </c>
       <c r="C579" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D579" t="n">
-        <v>92</v>
+        <v>51</v>
       </c>
       <c r="E579" t="inlineStr">
         <is>
@@ -14828,16 +14828,16 @@
       </c>
       <c r="B580" t="inlineStr">
         <is>
-          <t>22:31</t>
+          <t>21:59</t>
         </is>
       </c>
       <c r="C580" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D580" t="n">
-        <v>103</v>
+        <v>71</v>
       </c>
       <c r="E580" t="inlineStr">
         <is>
@@ -14848,23 +14848,273 @@
     <row r="581">
       <c r="A581" t="inlineStr">
         <is>
+          <t>21:01:13</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D581" t="n">
+        <v>59</v>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>21:01:13</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>22:01</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D582" t="n">
+        <v>60</v>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>21:01:13</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>22:14</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D583" t="n">
+        <v>73</v>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
           <t>20:48:48</t>
         </is>
       </c>
-      <c r="B581" t="inlineStr">
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>22:16</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D584" t="n">
+        <v>88</v>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>21:01:13</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>22:19</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D585" t="n">
+        <v>78</v>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>20:48:48</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>22:20</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D586" t="n">
+        <v>92</v>
+      </c>
+      <c r="E586" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>21:01:13</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>22:21</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D587" t="n">
+        <v>80</v>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>21:01:13</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>22:31</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D588" t="n">
+        <v>90</v>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>20:48:48</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
         <is>
           <t>22:41</t>
         </is>
       </c>
-      <c r="C581" t="inlineStr">
+      <c r="C589" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D581" t="n">
+      <c r="D589" t="n">
         <v>113</v>
       </c>
-      <c r="E581" t="inlineStr">
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>21:01:13</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>22:43</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D590" t="n">
+        <v>102</v>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>21:01:13</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>22:57</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D591" t="n">
+        <v>116</v>
+      </c>
+      <c r="E591" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -14881,7 +15131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14894,14 +15144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:48:48</t>
+          <t>Última actualización: 21:01:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 66</t>
+          <t>Total filas: 67</t>
         </is>
       </c>
     </row>
@@ -16577,6 +16827,31 @@
         <v>115</v>
       </c>
       <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>21:01:13</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>22:57</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>116</v>
+      </c>
+      <c r="E72" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -16593,7 +16868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16606,14 +16881,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:48:48</t>
+          <t>Última actualización: 21:01:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 77</t>
+          <t>Total filas: 79</t>
         </is>
       </c>
     </row>
@@ -18472,7 +18747,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>20:48:48</t>
+          <t>21:01:13</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -18486,7 +18761,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -18547,23 +18822,73 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
+          <t>21:01:13</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>22:21</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>80</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
           <t>20:48:48</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>22:25</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D82" t="n">
+      <c r="D83" t="n">
         <v>97</v>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>21:01:13</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>85</v>
+      </c>
+      <c r="E84" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>